<commit_message>
added variables and fixed issue with MICE implementation
</commit_message>
<xml_diff>
--- a/graphs/PCR_Retention_National.xlsx
+++ b/graphs/PCR_Retention_National.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="19">
   <si>
     <t>year</t>
   </si>
@@ -52,7 +52,13 @@
     <t>Men Doctor</t>
   </si>
   <si>
+    <t>Women Doctor</t>
+  </si>
+  <si>
     <t>Men Masters</t>
+  </si>
+  <si>
+    <t>Women Masters</t>
   </si>
   <si>
     <t>White</t>
@@ -422,7 +428,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G141"/>
+  <dimension ref="A1:G169"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -453,19 +459,19 @@
         <v>2010</v>
       </c>
       <c r="B2">
-        <v>1.228134110787172</v>
+        <v>0.960597302504817</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
       </c>
       <c r="E2">
-        <v>1685</v>
+        <v>2956</v>
       </c>
       <c r="F2">
-        <v>1372</v>
+        <v>5027</v>
       </c>
       <c r="G2">
-        <v>3590</v>
+        <v>25245</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -473,22 +479,22 @@
         <v>2011</v>
       </c>
       <c r="B3">
-        <v>0.7943229409027455</v>
+        <v>0.6572472126105344</v>
       </c>
       <c r="C3">
-        <v>0.9729805013927577</v>
+        <v>0.9473955238661121</v>
       </c>
       <c r="D3" t="s">
         <v>7</v>
       </c>
       <c r="E3">
-        <v>1707</v>
+        <v>3012</v>
       </c>
       <c r="F3">
-        <v>2149</v>
+        <v>5353</v>
       </c>
       <c r="G3">
-        <v>3610</v>
+        <v>26258</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -496,22 +502,22 @@
         <v>2012</v>
       </c>
       <c r="B4">
-        <v>0.7782846715328468</v>
+        <v>0.65517459915077</v>
       </c>
       <c r="C4">
-        <v>0.9869806094182826</v>
+        <v>0.9104272983471704</v>
       </c>
       <c r="D4" t="s">
         <v>7</v>
       </c>
       <c r="E4">
-        <v>1706</v>
+        <v>3255</v>
       </c>
       <c r="F4">
-        <v>2192</v>
+        <v>5226</v>
       </c>
       <c r="G4">
-        <v>3771</v>
+        <v>25877</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -519,22 +525,22 @@
         <v>2013</v>
       </c>
       <c r="B5">
-        <v>0.7544910179640718</v>
+        <v>0.6672210849539406</v>
       </c>
       <c r="C5">
-        <v>0.9610182975338106</v>
+        <v>0.951849132434208</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
       </c>
       <c r="E5">
-        <v>1638</v>
+        <v>3298</v>
       </c>
       <c r="F5">
-        <v>2171</v>
+        <v>5200</v>
       </c>
       <c r="G5">
-        <v>3794</v>
+        <v>26533</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -542,22 +548,22 @@
         <v>2014</v>
       </c>
       <c r="B6">
-        <v>0.7226851851851852</v>
+        <v>0.6299355484638007</v>
       </c>
       <c r="C6">
-        <v>0.9862941486557723</v>
+        <v>0.9513812987600346</v>
       </c>
       <c r="D6" t="s">
         <v>7</v>
       </c>
       <c r="E6">
-        <v>1561</v>
+        <v>3257</v>
       </c>
       <c r="F6">
-        <v>2160</v>
+        <v>5206</v>
       </c>
       <c r="G6">
-        <v>3863</v>
+        <v>27192</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -565,22 +571,22 @@
         <v>2015</v>
       </c>
       <c r="B7">
-        <v>0.7388475836431226</v>
+        <v>0.6268647553563754</v>
       </c>
       <c r="C7">
-        <v>0.9823971006989386</v>
+        <v>0.9225507502206531</v>
       </c>
       <c r="D7" t="s">
         <v>7</v>
       </c>
       <c r="E7">
-        <v>1590</v>
+        <v>3340</v>
       </c>
       <c r="F7">
-        <v>2152</v>
+        <v>5575</v>
       </c>
       <c r="G7">
-        <v>4015</v>
+        <v>27321</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -588,22 +594,22 @@
         <v>2016</v>
       </c>
       <c r="B8">
-        <v>0.7462422634836428</v>
+        <v>0.6174329842002485</v>
       </c>
       <c r="C8">
-        <v>0.9469489414694894</v>
+        <v>0.9368617546941913</v>
       </c>
       <c r="D8" t="s">
         <v>7</v>
       </c>
       <c r="E8">
-        <v>1688</v>
+        <v>3309</v>
       </c>
       <c r="F8">
-        <v>2262</v>
+        <v>5508</v>
       </c>
       <c r="G8">
-        <v>3956</v>
+        <v>27795</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -611,22 +617,22 @@
         <v>2017</v>
       </c>
       <c r="B9">
-        <v>0.5280105866784296</v>
+        <v>0.4194793799356537</v>
       </c>
       <c r="C9">
-        <v>0.9661274014155713</v>
+        <v>0.9210649397373628</v>
       </c>
       <c r="D9" t="s">
         <v>7</v>
       </c>
       <c r="E9">
-        <v>1197</v>
+        <v>3322</v>
       </c>
       <c r="F9">
-        <v>2267</v>
+        <v>5816</v>
       </c>
       <c r="G9">
-        <v>4025</v>
+        <v>28095</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -634,22 +640,22 @@
         <v>2018</v>
       </c>
       <c r="B10">
-        <v>0.2678185745140389</v>
+        <v>0.2111711084015561</v>
       </c>
       <c r="C10">
-        <v>0.9008695652173913</v>
+        <v>0.9158213205196655</v>
       </c>
       <c r="D10" t="s">
         <v>7</v>
       </c>
       <c r="E10">
-        <v>620</v>
+        <v>3626</v>
       </c>
       <c r="F10">
-        <v>2315</v>
+        <v>5771</v>
       </c>
       <c r="G10">
-        <v>3829</v>
+        <v>27875</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -660,19 +666,19 @@
         <v>0</v>
       </c>
       <c r="C11">
-        <v>0.9579524680073126</v>
+        <v>0.9225829596412556</v>
       </c>
       <c r="D11" t="s">
         <v>7</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>3390</v>
       </c>
       <c r="F11">
-        <v>2116</v>
+        <v>5636</v>
       </c>
       <c r="G11">
-        <v>3871</v>
+        <v>27963</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -683,19 +689,19 @@
         <v>0</v>
       </c>
       <c r="C12">
-        <v>0.9323172306897443</v>
+        <v>0.9284769159246147</v>
       </c>
       <c r="D12" t="s">
         <v>7</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>3414</v>
       </c>
       <c r="F12">
-        <v>2087</v>
+        <v>4827</v>
       </c>
       <c r="G12">
-        <v>3681</v>
+        <v>27376</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -706,19 +712,19 @@
         <v>0</v>
       </c>
       <c r="C13">
-        <v>0.971746807932627</v>
+        <v>0.9558007013442431</v>
       </c>
       <c r="D13" t="s">
         <v>7</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>3263</v>
       </c>
       <c r="F13">
-        <v>2144</v>
+        <v>5945</v>
       </c>
       <c r="G13">
-        <v>3828</v>
+        <v>28848</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -729,19 +735,19 @@
         <v>0</v>
       </c>
       <c r="C14">
-        <v>0.9655172413793104</v>
+        <v>0.9286952301719357</v>
       </c>
       <c r="D14" t="s">
         <v>7</v>
       </c>
       <c r="E14">
-        <v>0</v>
+        <v>3534</v>
       </c>
       <c r="F14">
-        <v>2390</v>
+        <v>5752</v>
       </c>
       <c r="G14">
-        <v>3927</v>
+        <v>29009</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -752,19 +758,19 @@
         <v>0</v>
       </c>
       <c r="C15">
-        <v>1.016297428062134</v>
+        <v>0.9463270019649075</v>
       </c>
       <c r="D15" t="s">
         <v>7</v>
       </c>
       <c r="E15">
-        <v>0</v>
+        <v>3637</v>
       </c>
       <c r="F15">
-        <v>1648</v>
+        <v>6031</v>
       </c>
       <c r="G15">
-        <v>4211</v>
+        <v>29846</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -772,19 +778,19 @@
         <v>2010</v>
       </c>
       <c r="B16">
-        <v>1.11716621253406</v>
+        <v>0.9551173481732398</v>
       </c>
       <c r="D16" t="s">
         <v>8</v>
       </c>
       <c r="E16">
-        <v>1230</v>
+        <v>2345</v>
       </c>
       <c r="F16">
-        <v>1101</v>
+        <v>4006</v>
       </c>
       <c r="G16">
-        <v>2842</v>
+        <v>20208</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -792,22 +798,22 @@
         <v>2011</v>
       </c>
       <c r="B17">
-        <v>0.7238590410167534</v>
+        <v>0.6485617869194922</v>
       </c>
       <c r="C17">
-        <v>0.9560168895144264</v>
+        <v>0.948535233570863</v>
       </c>
       <c r="D17" t="s">
         <v>8</v>
       </c>
       <c r="E17">
-        <v>1253</v>
+        <v>2403</v>
       </c>
       <c r="F17">
-        <v>1731</v>
+        <v>4260</v>
       </c>
       <c r="G17">
-        <v>2876</v>
+        <v>21025</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -815,22 +821,22 @@
         <v>2012</v>
       </c>
       <c r="B18">
-        <v>0.7146860986547086</v>
+        <v>0.6449924668939815</v>
       </c>
       <c r="C18">
-        <v>0.9690542420027817</v>
+        <v>0.9088228299643282</v>
       </c>
       <c r="D18" t="s">
         <v>8</v>
       </c>
       <c r="E18">
-        <v>1275</v>
+        <v>2588</v>
       </c>
       <c r="F18">
-        <v>1784</v>
+        <v>4180</v>
       </c>
       <c r="G18">
-        <v>3018</v>
+        <v>20700</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -838,22 +844,22 @@
         <v>2013</v>
       </c>
       <c r="B19">
-        <v>0.686541737649063</v>
+        <v>0.6548878205128205</v>
       </c>
       <c r="C19">
-        <v>0.9466534128561962</v>
+        <v>0.9563768115942028</v>
       </c>
       <c r="D19" t="s">
         <v>8</v>
       </c>
       <c r="E19">
-        <v>1209</v>
+        <v>2653</v>
       </c>
       <c r="F19">
-        <v>1761</v>
+        <v>4171</v>
       </c>
       <c r="G19">
-        <v>3055</v>
+        <v>21315</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -861,22 +867,22 @@
         <v>2014</v>
       </c>
       <c r="B20">
-        <v>0.6586345381526104</v>
+        <v>0.62435029138447</v>
       </c>
       <c r="C20">
-        <v>0.9741407528641571</v>
+        <v>0.9505043396669013</v>
       </c>
       <c r="D20" t="s">
         <v>8</v>
       </c>
       <c r="E20">
-        <v>1148</v>
+        <v>2587</v>
       </c>
       <c r="F20">
-        <v>1743</v>
+        <v>4129</v>
       </c>
       <c r="G20">
-        <v>3118</v>
+        <v>21802</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -884,22 +890,22 @@
         <v>2015</v>
       </c>
       <c r="B21">
-        <v>0.6763509587449158</v>
+        <v>0.6220024914356899</v>
       </c>
       <c r="C21">
-        <v>0.9701731879409878</v>
+        <v>0.921566828731309</v>
       </c>
       <c r="D21" t="s">
         <v>8</v>
       </c>
       <c r="E21">
-        <v>1164</v>
+        <v>2638</v>
       </c>
       <c r="F21">
-        <v>1721</v>
+        <v>4398</v>
       </c>
       <c r="G21">
-        <v>3246</v>
+        <v>21852</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -907,22 +913,22 @@
         <v>2016</v>
       </c>
       <c r="B22">
-        <v>0.6839492553778268</v>
+        <v>0.6129251187693235</v>
       </c>
       <c r="C22">
-        <v>0.9306839186691312</v>
+        <v>0.9341021416803954</v>
       </c>
       <c r="D22" t="s">
         <v>8</v>
       </c>
       <c r="E22">
-        <v>1240</v>
+        <v>2625</v>
       </c>
       <c r="F22">
-        <v>1813</v>
+        <v>4317</v>
       </c>
       <c r="G22">
-        <v>3192</v>
+        <v>22104</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -930,22 +936,22 @@
         <v>2017</v>
       </c>
       <c r="B23">
-        <v>0.4914127423822715</v>
+        <v>0.4146523425843032</v>
       </c>
       <c r="C23">
-        <v>0.9598997493734336</v>
+        <v>0.9197882736156352</v>
       </c>
       <c r="D23" t="s">
         <v>8</v>
       </c>
       <c r="E23">
-        <v>887</v>
+        <v>2632</v>
       </c>
       <c r="F23">
-        <v>1805</v>
+        <v>4546</v>
       </c>
       <c r="G23">
-        <v>3255</v>
+        <v>22245</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -953,22 +959,22 @@
         <v>2018</v>
       </c>
       <c r="B24">
-        <v>0.2474114441416894</v>
+        <v>0.2081789894799229</v>
       </c>
       <c r="C24">
-        <v>0.8835637480798771</v>
+        <v>0.9100022476961115</v>
       </c>
       <c r="D24" t="s">
         <v>8</v>
       </c>
       <c r="E24">
-        <v>454</v>
+        <v>2815</v>
       </c>
       <c r="F24">
-        <v>1835</v>
+        <v>4541</v>
       </c>
       <c r="G24">
-        <v>3066</v>
+        <v>21969</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -979,19 +985,19 @@
         <v>0</v>
       </c>
       <c r="C25">
-        <v>0.9527071102413568</v>
+        <v>0.9239837953479904</v>
       </c>
       <c r="D25" t="s">
         <v>8</v>
       </c>
       <c r="E25">
-        <v>0</v>
+        <v>2687</v>
       </c>
       <c r="F25">
-        <v>1641</v>
+        <v>4411</v>
       </c>
       <c r="G25">
-        <v>3100</v>
+        <v>22023</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -1002,19 +1008,19 @@
         <v>0</v>
       </c>
       <c r="C26">
-        <v>0.9132258064516129</v>
+        <v>0.9244880352358897</v>
       </c>
       <c r="D26" t="s">
         <v>8</v>
       </c>
       <c r="E26">
-        <v>0</v>
+        <v>2671</v>
       </c>
       <c r="F26">
-        <v>1605</v>
+        <v>3654</v>
       </c>
       <c r="G26">
-        <v>2894</v>
+        <v>21343</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -1025,19 +1031,19 @@
         <v>0</v>
       </c>
       <c r="C27">
-        <v>0.9557705597788528</v>
+        <v>0.9493510752940074</v>
       </c>
       <c r="D27" t="s">
         <v>8</v>
       </c>
       <c r="E27">
-        <v>0</v>
+        <v>2570</v>
       </c>
       <c r="F27">
-        <v>1600</v>
+        <v>4284</v>
       </c>
       <c r="G27">
-        <v>2981</v>
+        <v>21976</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -1048,19 +1054,19 @@
         <v>0</v>
       </c>
       <c r="C28">
-        <v>0.9446494464944649</v>
+        <v>0.9285584273753186</v>
       </c>
       <c r="D28" t="s">
         <v>8</v>
       </c>
       <c r="E28">
-        <v>0</v>
+        <v>2748</v>
       </c>
       <c r="F28">
-        <v>1783</v>
+        <v>4141</v>
       </c>
       <c r="G28">
-        <v>2974</v>
+        <v>21799</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -1071,19 +1077,19 @@
         <v>0</v>
       </c>
       <c r="C29">
-        <v>1.010423671822461</v>
+        <v>0.9472452864810312</v>
       </c>
       <c r="D29" t="s">
         <v>8</v>
       </c>
       <c r="E29">
-        <v>0</v>
+        <v>2810</v>
       </c>
       <c r="F29">
-        <v>1215</v>
+        <v>4346</v>
       </c>
       <c r="G29">
-        <v>3175</v>
+        <v>22185</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -1091,19 +1097,19 @@
         <v>2010</v>
       </c>
       <c r="B30">
-        <v>1.088560885608856</v>
+        <v>0.9820245979186376</v>
       </c>
       <c r="D30" t="s">
         <v>9</v>
       </c>
       <c r="E30">
-        <v>295</v>
+        <v>611</v>
       </c>
       <c r="F30">
-        <v>271</v>
+        <v>1021</v>
       </c>
       <c r="G30">
-        <v>748</v>
+        <v>5037</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -1111,22 +1117,22 @@
         <v>2011</v>
       </c>
       <c r="B31">
-        <v>0.722488038277512</v>
+        <v>0.6914556962025317</v>
       </c>
       <c r="C31">
-        <v>0.9197860962566845</v>
+        <v>0.9428231089934485</v>
       </c>
       <c r="D31" t="s">
         <v>9</v>
       </c>
       <c r="E31">
-        <v>302</v>
+        <v>609</v>
       </c>
       <c r="F31">
-        <v>418</v>
+        <v>1093</v>
       </c>
       <c r="G31">
-        <v>734</v>
+        <v>5233</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -1134,22 +1140,22 @@
         <v>2012</v>
       </c>
       <c r="B32">
-        <v>0.7230392156862745</v>
+        <v>0.6957070707070707</v>
       </c>
       <c r="C32">
-        <v>0.9700272479564033</v>
+        <v>0.9168736862220523</v>
       </c>
       <c r="D32" t="s">
         <v>9</v>
       </c>
       <c r="E32">
-        <v>295</v>
+        <v>667</v>
       </c>
       <c r="F32">
-        <v>408</v>
+        <v>1046</v>
       </c>
       <c r="G32">
-        <v>753</v>
+        <v>5177</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -1157,22 +1163,22 @@
         <v>2013</v>
       </c>
       <c r="B33">
-        <v>0.7146341463414634</v>
+        <v>0.7160532994923858</v>
       </c>
       <c r="C33">
-        <v>0.9335989375830013</v>
+        <v>0.9337454124010044</v>
       </c>
       <c r="D33" t="s">
         <v>9</v>
       </c>
       <c r="E33">
-        <v>293</v>
+        <v>645</v>
       </c>
       <c r="F33">
-        <v>410</v>
+        <v>1029</v>
       </c>
       <c r="G33">
-        <v>739</v>
+        <v>5218</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -1180,22 +1186,22 @@
         <v>2014</v>
       </c>
       <c r="B34">
-        <v>0.6642685851318945</v>
+        <v>0.651538227231191</v>
       </c>
       <c r="C34">
-        <v>0.9607577807848444</v>
+        <v>0.9549635875814488</v>
       </c>
       <c r="D34" t="s">
         <v>9</v>
       </c>
       <c r="E34">
-        <v>277</v>
+        <v>670</v>
       </c>
       <c r="F34">
-        <v>417</v>
+        <v>1077</v>
       </c>
       <c r="G34">
-        <v>745</v>
+        <v>5390</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -1203,22 +1209,22 @@
         <v>2015</v>
       </c>
       <c r="B35">
-        <v>0.654292343387471</v>
+        <v>0.6449927431059507</v>
       </c>
       <c r="C35">
-        <v>0.9583892617449664</v>
+        <v>0.926530612244898</v>
       </c>
       <c r="D35" t="s">
         <v>9</v>
       </c>
       <c r="E35">
-        <v>282</v>
+        <v>702</v>
       </c>
       <c r="F35">
-        <v>431</v>
+        <v>1177</v>
       </c>
       <c r="G35">
-        <v>769</v>
+        <v>5469</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -1226,22 +1232,22 @@
         <v>2016</v>
       </c>
       <c r="B36">
-        <v>0.6770601336302895</v>
+        <v>0.6338647608576141</v>
       </c>
       <c r="C36">
-        <v>0.9427828348504551</v>
+        <v>0.947888096544158</v>
       </c>
       <c r="D36" t="s">
         <v>9</v>
       </c>
       <c r="E36">
-        <v>304</v>
+        <v>684</v>
       </c>
       <c r="F36">
-        <v>449</v>
+        <v>1191</v>
       </c>
       <c r="G36">
-        <v>764</v>
+        <v>5691</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -1249,22 +1255,22 @@
         <v>2017</v>
       </c>
       <c r="B37">
-        <v>0.4632034632034632</v>
+        <v>0.437008940666486</v>
       </c>
       <c r="C37">
-        <v>0.9293193717277487</v>
+        <v>0.9260235459497452</v>
       </c>
       <c r="D37" t="s">
         <v>9</v>
       </c>
       <c r="E37">
-        <v>214</v>
+        <v>690</v>
       </c>
       <c r="F37">
-        <v>462</v>
+        <v>1270</v>
       </c>
       <c r="G37">
-        <v>770</v>
+        <v>5850</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -1272,22 +1278,22 @@
         <v>2018</v>
       </c>
       <c r="B38">
-        <v>0.2458333333333333</v>
+        <v>0.2220134228187919</v>
       </c>
       <c r="C38">
-        <v>0.9116883116883117</v>
+        <v>0.9379487179487179</v>
       </c>
       <c r="D38" t="s">
         <v>9</v>
       </c>
       <c r="E38">
-        <v>118</v>
+        <v>811</v>
       </c>
       <c r="F38">
-        <v>480</v>
+        <v>1230</v>
       </c>
       <c r="G38">
-        <v>763</v>
+        <v>5906</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -1298,19 +1304,19 @@
         <v>0</v>
       </c>
       <c r="C39">
-        <v>0.926605504587156</v>
+        <v>0.9173721639011175</v>
       </c>
       <c r="D39" t="s">
         <v>9</v>
       </c>
       <c r="E39">
-        <v>0</v>
+        <v>703</v>
       </c>
       <c r="F39">
-        <v>475</v>
+        <v>1225</v>
       </c>
       <c r="G39">
-        <v>771</v>
+        <v>5940</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -1321,19 +1327,19 @@
         <v>0</v>
       </c>
       <c r="C40">
-        <v>0.9468223086900129</v>
+        <v>0.9432659932659933</v>
       </c>
       <c r="D40" t="s">
         <v>9</v>
       </c>
       <c r="E40">
-        <v>0</v>
+        <v>743</v>
       </c>
       <c r="F40">
-        <v>482</v>
+        <v>1173</v>
       </c>
       <c r="G40">
-        <v>787</v>
+        <v>6033</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -1344,19 +1350,19 @@
         <v>0</v>
       </c>
       <c r="C41">
-        <v>0.9695044472681067</v>
+        <v>0.9786176031824962</v>
       </c>
       <c r="D41" t="s">
         <v>9</v>
       </c>
       <c r="E41">
-        <v>0</v>
+        <v>693</v>
       </c>
       <c r="F41">
-        <v>544</v>
+        <v>1661</v>
       </c>
       <c r="G41">
-        <v>847</v>
+        <v>6872</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -1367,19 +1373,19 @@
         <v>0</v>
       </c>
       <c r="C42">
-        <v>0.9822904368358913</v>
+        <v>0.9291327124563445</v>
       </c>
       <c r="D42" t="s">
         <v>9</v>
       </c>
       <c r="E42">
-        <v>0</v>
+        <v>786</v>
       </c>
       <c r="F42">
-        <v>607</v>
+        <v>1611</v>
       </c>
       <c r="G42">
-        <v>953</v>
+        <v>7210</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -1390,19 +1396,19 @@
         <v>0</v>
       </c>
       <c r="C43">
-        <v>0.9842602308499475</v>
+        <v>0.9435506241331484</v>
       </c>
       <c r="D43" t="s">
         <v>9</v>
       </c>
       <c r="E43">
-        <v>0</v>
+        <v>827</v>
       </c>
       <c r="F43">
-        <v>433</v>
+        <v>1685</v>
       </c>
       <c r="G43">
-        <v>1036</v>
+        <v>7661</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -1413,7 +1419,7 @@
         <v>10</v>
       </c>
       <c r="E44">
-        <v>1685</v>
+        <v>1384</v>
       </c>
       <c r="F44">
         <v>0</v>
@@ -1430,7 +1436,7 @@
         <v>10</v>
       </c>
       <c r="E45">
-        <v>1707</v>
+        <v>1500</v>
       </c>
       <c r="F45">
         <v>0</v>
@@ -1447,7 +1453,7 @@
         <v>10</v>
       </c>
       <c r="E46">
-        <v>1706</v>
+        <v>1615</v>
       </c>
       <c r="F46">
         <v>0</v>
@@ -1464,7 +1470,7 @@
         <v>10</v>
       </c>
       <c r="E47">
-        <v>1638</v>
+        <v>1579</v>
       </c>
       <c r="F47">
         <v>0</v>
@@ -1481,7 +1487,7 @@
         <v>10</v>
       </c>
       <c r="E48">
-        <v>1561</v>
+        <v>1609</v>
       </c>
       <c r="F48">
         <v>0</v>
@@ -1498,7 +1504,7 @@
         <v>10</v>
       </c>
       <c r="E49">
-        <v>1590</v>
+        <v>1672</v>
       </c>
       <c r="F49">
         <v>0</v>
@@ -1512,16 +1518,16 @@
         <v>2016</v>
       </c>
       <c r="B50">
-        <v>2.364145658263305</v>
+        <v>2.202321724709785</v>
       </c>
       <c r="D50" t="s">
         <v>10</v>
       </c>
       <c r="E50">
-        <v>1688</v>
+        <v>1653</v>
       </c>
       <c r="F50">
-        <v>714</v>
+        <v>0</v>
       </c>
       <c r="G50">
         <v>0</v>
@@ -1532,19 +1538,19 @@
         <v>2017</v>
       </c>
       <c r="B51">
-        <v>0.8537803138373752</v>
+        <v>0.7661122661122661</v>
       </c>
       <c r="D51" t="s">
         <v>10</v>
       </c>
       <c r="E51">
-        <v>1197</v>
+        <v>1687</v>
       </c>
       <c r="F51">
-        <v>1402</v>
+        <v>2412</v>
       </c>
       <c r="G51">
-        <v>3842</v>
+        <v>12780</v>
       </c>
     </row>
     <row r="52" spans="1:7">
@@ -1552,22 +1558,22 @@
         <v>2018</v>
       </c>
       <c r="B52">
-        <v>0.3006789524733269</v>
+        <v>0.2606819763395964</v>
       </c>
       <c r="C52">
-        <v>0.9190525767829255</v>
+        <v>0.9413145539906104</v>
       </c>
       <c r="D52" t="s">
         <v>10</v>
       </c>
       <c r="E52">
-        <v>620</v>
+        <v>1732</v>
       </c>
       <c r="F52">
-        <v>2062</v>
+        <v>2398</v>
       </c>
       <c r="G52">
-        <v>3651</v>
+        <v>12696</v>
       </c>
     </row>
     <row r="53" spans="1:7">
@@ -1578,19 +1584,19 @@
         <v>0</v>
       </c>
       <c r="C53">
-        <v>0.9660367022733498</v>
+        <v>0.9577819785759294</v>
       </c>
       <c r="D53" t="s">
         <v>10</v>
       </c>
       <c r="E53">
-        <v>0</v>
+        <v>1722</v>
       </c>
       <c r="F53">
-        <v>1882</v>
+        <v>2375</v>
       </c>
       <c r="G53">
-        <v>3639</v>
+        <v>12813</v>
       </c>
     </row>
     <row r="54" spans="1:7">
@@ -1601,19 +1607,19 @@
         <v>0</v>
       </c>
       <c r="C54">
-        <v>0.9530090684253916</v>
+        <v>0.9566846171856708</v>
       </c>
       <c r="D54" t="s">
         <v>10</v>
       </c>
       <c r="E54">
-        <v>0</v>
+        <v>1647</v>
       </c>
       <c r="F54">
-        <v>1855</v>
+        <v>1979</v>
       </c>
       <c r="G54">
-        <v>3480</v>
+        <v>12590</v>
       </c>
     </row>
     <row r="55" spans="1:7">
@@ -1624,19 +1630,19 @@
         <v>0</v>
       </c>
       <c r="C55">
-        <v>0.992816091954023</v>
+        <v>0.9861000794281175</v>
       </c>
       <c r="D55" t="s">
         <v>10</v>
       </c>
       <c r="E55">
-        <v>0</v>
+        <v>1627</v>
       </c>
       <c r="F55">
-        <v>1921</v>
+        <v>2479</v>
       </c>
       <c r="G55">
-        <v>3625</v>
+        <v>13267</v>
       </c>
     </row>
     <row r="56" spans="1:7">
@@ -1647,19 +1653,19 @@
         <v>0</v>
       </c>
       <c r="C56">
-        <v>0.9806896551724138</v>
+        <v>0.9694731288158589</v>
       </c>
       <c r="D56" t="s">
         <v>10</v>
       </c>
       <c r="E56">
-        <v>0</v>
+        <v>1812</v>
       </c>
       <c r="F56">
-        <v>2153</v>
+        <v>2449</v>
       </c>
       <c r="G56">
-        <v>3704</v>
+        <v>13499</v>
       </c>
     </row>
     <row r="57" spans="1:7">
@@ -1670,19 +1676,19 @@
         <v>0</v>
       </c>
       <c r="C57">
-        <v>1.047246220302376</v>
+        <v>0.979628120601526</v>
       </c>
       <c r="D57" t="s">
         <v>10</v>
       </c>
       <c r="E57">
-        <v>0</v>
+        <v>1873</v>
       </c>
       <c r="F57">
-        <v>1492</v>
+        <v>2565</v>
       </c>
       <c r="G57">
-        <v>4025</v>
+        <v>13916</v>
       </c>
     </row>
     <row r="58" spans="1:7">
@@ -1693,7 +1699,7 @@
         <v>11</v>
       </c>
       <c r="E58">
-        <v>1230</v>
+        <v>1127</v>
       </c>
       <c r="F58">
         <v>0</v>
@@ -1710,7 +1716,7 @@
         <v>11</v>
       </c>
       <c r="E59">
-        <v>1253</v>
+        <v>1237</v>
       </c>
       <c r="F59">
         <v>0</v>
@@ -1727,7 +1733,7 @@
         <v>11</v>
       </c>
       <c r="E60">
-        <v>1275</v>
+        <v>1301</v>
       </c>
       <c r="F60">
         <v>0</v>
@@ -1744,7 +1750,7 @@
         <v>11</v>
       </c>
       <c r="E61">
-        <v>1209</v>
+        <v>1274</v>
       </c>
       <c r="F61">
         <v>0</v>
@@ -1761,7 +1767,7 @@
         <v>11</v>
       </c>
       <c r="E62">
-        <v>1148</v>
+        <v>1317</v>
       </c>
       <c r="F62">
         <v>0</v>
@@ -1778,7 +1784,7 @@
         <v>11</v>
       </c>
       <c r="E63">
-        <v>1164</v>
+        <v>1338</v>
       </c>
       <c r="F63">
         <v>0</v>
@@ -1792,16 +1798,16 @@
         <v>2016</v>
       </c>
       <c r="B64">
-        <v>2.190812720848057</v>
+        <v>2.234234234234234</v>
       </c>
       <c r="D64" t="s">
         <v>11</v>
       </c>
       <c r="E64">
-        <v>1240</v>
+        <v>1343</v>
       </c>
       <c r="F64">
-        <v>566</v>
+        <v>0</v>
       </c>
       <c r="G64">
         <v>0</v>
@@ -1812,19 +1818,19 @@
         <v>2017</v>
       </c>
       <c r="B65">
-        <v>0.8063636363636364</v>
+        <v>0.7726427622841966</v>
       </c>
       <c r="D65" t="s">
         <v>11</v>
       </c>
       <c r="E65">
-        <v>887</v>
+        <v>1391</v>
       </c>
       <c r="F65">
-        <v>1100</v>
+        <v>1887</v>
       </c>
       <c r="G65">
-        <v>3111</v>
+        <v>10174</v>
       </c>
     </row>
     <row r="66" spans="1:7">
@@ -1832,22 +1838,22 @@
         <v>2018</v>
       </c>
       <c r="B66">
-        <v>0.2804200123533045</v>
+        <v>0.2631016042780749</v>
       </c>
       <c r="C66">
-        <v>0.9016393442622951</v>
+        <v>0.9356202083742874</v>
       </c>
       <c r="D66" t="s">
         <v>11</v>
       </c>
       <c r="E66">
-        <v>454</v>
+        <v>1364</v>
       </c>
       <c r="F66">
-        <v>1619</v>
+        <v>1878</v>
       </c>
       <c r="G66">
-        <v>2925</v>
+        <v>10033</v>
       </c>
     </row>
     <row r="67" spans="1:7">
@@ -1858,19 +1864,19 @@
         <v>0</v>
       </c>
       <c r="C67">
-        <v>0.9593162393162393</v>
+        <v>0.9603309080035881</v>
       </c>
       <c r="D67" t="s">
         <v>11</v>
       </c>
       <c r="E67">
-        <v>0</v>
+        <v>1378</v>
       </c>
       <c r="F67">
-        <v>1446</v>
+        <v>1845</v>
       </c>
       <c r="G67">
-        <v>2908</v>
+        <v>10102</v>
       </c>
     </row>
     <row r="68" spans="1:7">
@@ -1881,19 +1887,19 @@
         <v>0</v>
       </c>
       <c r="C68">
-        <v>0.9339752407152683</v>
+        <v>0.9538705206889725</v>
       </c>
       <c r="D68" t="s">
         <v>11</v>
       </c>
       <c r="E68">
-        <v>0</v>
+        <v>1311</v>
       </c>
       <c r="F68">
-        <v>1412</v>
+        <v>1494</v>
       </c>
       <c r="G68">
-        <v>2731</v>
+        <v>9819</v>
       </c>
     </row>
     <row r="69" spans="1:7">
@@ -1904,19 +1910,19 @@
         <v>0</v>
       </c>
       <c r="C69">
-        <v>0.9783961918711095</v>
+        <v>0.9829921580609023</v>
       </c>
       <c r="D69" t="s">
         <v>11</v>
       </c>
       <c r="E69">
-        <v>0</v>
+        <v>1307</v>
       </c>
       <c r="F69">
-        <v>1417</v>
+        <v>1774</v>
       </c>
       <c r="G69">
-        <v>2819</v>
+        <v>10119</v>
       </c>
     </row>
     <row r="70" spans="1:7">
@@ -1927,19 +1933,19 @@
         <v>0</v>
       </c>
       <c r="C70">
-        <v>0.9567222419297623</v>
+        <v>0.9706492736436407</v>
       </c>
       <c r="D70" t="s">
         <v>11</v>
       </c>
       <c r="E70">
-        <v>0</v>
+        <v>1433</v>
       </c>
       <c r="F70">
-        <v>1584</v>
+        <v>1763</v>
       </c>
       <c r="G70">
-        <v>2788</v>
+        <v>10152</v>
       </c>
     </row>
     <row r="71" spans="1:7">
@@ -1950,19 +1956,19 @@
         <v>0</v>
       </c>
       <c r="C71">
-        <v>1.047704447632712</v>
+        <v>0.9839440504334122</v>
       </c>
       <c r="D71" t="s">
         <v>11</v>
       </c>
       <c r="E71">
-        <v>0</v>
+        <v>1476</v>
       </c>
       <c r="F71">
-        <v>1084</v>
+        <v>1837</v>
       </c>
       <c r="G71">
-        <v>3027</v>
+        <v>10350</v>
       </c>
     </row>
     <row r="72" spans="1:7">
@@ -1973,7 +1979,7 @@
         <v>12</v>
       </c>
       <c r="E72">
-        <v>1230</v>
+        <v>257</v>
       </c>
       <c r="F72">
         <v>0</v>
@@ -1990,7 +1996,7 @@
         <v>12</v>
       </c>
       <c r="E73">
-        <v>1253</v>
+        <v>263</v>
       </c>
       <c r="F73">
         <v>0</v>
@@ -2007,7 +2013,7 @@
         <v>12</v>
       </c>
       <c r="E74">
-        <v>1275</v>
+        <v>314</v>
       </c>
       <c r="F74">
         <v>0</v>
@@ -2024,7 +2030,7 @@
         <v>12</v>
       </c>
       <c r="E75">
-        <v>1209</v>
+        <v>305</v>
       </c>
       <c r="F75">
         <v>0</v>
@@ -2041,7 +2047,7 @@
         <v>12</v>
       </c>
       <c r="E76">
-        <v>1148</v>
+        <v>292</v>
       </c>
       <c r="F76">
         <v>0</v>
@@ -2058,7 +2064,7 @@
         <v>12</v>
       </c>
       <c r="E77">
-        <v>1164</v>
+        <v>334</v>
       </c>
       <c r="F77">
         <v>0</v>
@@ -2072,16 +2078,16 @@
         <v>2016</v>
       </c>
       <c r="B78">
-        <v>17.97101449275362</v>
+        <v>2.087619047619047</v>
       </c>
       <c r="D78" t="s">
         <v>12</v>
       </c>
       <c r="E78">
-        <v>1240</v>
+        <v>310</v>
       </c>
       <c r="F78">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="G78">
         <v>0</v>
@@ -2092,19 +2098,19 @@
         <v>2017</v>
       </c>
       <c r="B79">
-        <v>6.381294964028777</v>
+        <v>0.7425837320574162</v>
       </c>
       <c r="D79" t="s">
         <v>12</v>
       </c>
       <c r="E79">
-        <v>887</v>
+        <v>296</v>
       </c>
       <c r="F79">
-        <v>139</v>
+        <v>525</v>
       </c>
       <c r="G79">
-        <v>144</v>
+        <v>2606</v>
       </c>
     </row>
     <row r="80" spans="1:7">
@@ -2112,22 +2118,22 @@
         <v>2018</v>
       </c>
       <c r="B80">
-        <v>2.101851851851852</v>
+        <v>0.252063492063492</v>
       </c>
       <c r="C80">
-        <v>3.368055555555555</v>
+        <v>0.9635456638526477</v>
       </c>
       <c r="D80" t="s">
         <v>12</v>
       </c>
       <c r="E80">
-        <v>454</v>
+        <v>368</v>
       </c>
       <c r="F80">
-        <v>216</v>
+        <v>520</v>
       </c>
       <c r="G80">
-        <v>141</v>
+        <v>2663</v>
       </c>
     </row>
     <row r="81" spans="1:7">
@@ -2138,19 +2144,19 @@
         <v>0</v>
       </c>
       <c r="C81">
-        <v>3.773049645390071</v>
+        <v>0.9481787457754413</v>
       </c>
       <c r="D81" t="s">
         <v>12</v>
       </c>
       <c r="E81">
-        <v>0</v>
+        <v>344</v>
       </c>
       <c r="F81">
-        <v>195</v>
+        <v>530</v>
       </c>
       <c r="G81">
-        <v>192</v>
+        <v>2711</v>
       </c>
     </row>
     <row r="82" spans="1:7">
@@ -2161,19 +2167,19 @@
         <v>0</v>
       </c>
       <c r="C82">
-        <v>2.567708333333333</v>
+        <v>0.967170785687938</v>
       </c>
       <c r="D82" t="s">
         <v>12</v>
       </c>
       <c r="E82">
-        <v>0</v>
+        <v>336</v>
       </c>
       <c r="F82">
-        <v>193</v>
+        <v>485</v>
       </c>
       <c r="G82">
-        <v>163</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="83" spans="1:7">
@@ -2184,19 +2190,19 @@
         <v>0</v>
       </c>
       <c r="C83">
-        <v>2.742331288343558</v>
+        <v>0.9971129556116926</v>
       </c>
       <c r="D83" t="s">
         <v>12</v>
       </c>
       <c r="E83">
-        <v>0</v>
+        <v>320</v>
       </c>
       <c r="F83">
-        <v>183</v>
+        <v>705</v>
       </c>
       <c r="G83">
-        <v>162</v>
+        <v>3148</v>
       </c>
     </row>
     <row r="84" spans="1:7">
@@ -2207,19 +2213,19 @@
         <v>0</v>
       </c>
       <c r="C84">
-        <v>3.407407407407407</v>
+        <v>0.96569250317662</v>
       </c>
       <c r="D84" t="s">
         <v>12</v>
       </c>
       <c r="E84">
-        <v>0</v>
+        <v>379</v>
       </c>
       <c r="F84">
-        <v>199</v>
+        <v>686</v>
       </c>
       <c r="G84">
-        <v>186</v>
+        <v>3347</v>
       </c>
     </row>
     <row r="85" spans="1:7">
@@ -2230,154 +2236,121 @@
         <v>0</v>
       </c>
       <c r="C85">
-        <v>2.89247311827957</v>
+        <v>0.9665371974902898</v>
       </c>
       <c r="D85" t="s">
         <v>12</v>
       </c>
       <c r="E85">
-        <v>0</v>
+        <v>397</v>
       </c>
       <c r="F85">
-        <v>131</v>
+        <v>728</v>
       </c>
       <c r="G85">
-        <v>148</v>
+        <v>3566</v>
       </c>
     </row>
     <row r="86" spans="1:7">
       <c r="A86">
         <v>2010</v>
       </c>
-      <c r="B86">
-        <v>1.029411764705882</v>
-      </c>
       <c r="D86" t="s">
         <v>13</v>
       </c>
       <c r="E86">
-        <v>665</v>
+        <v>1218</v>
       </c>
       <c r="F86">
-        <v>646</v>
+        <v>0</v>
       </c>
       <c r="G86">
-        <v>1581</v>
+        <v>0</v>
       </c>
     </row>
     <row r="87" spans="1:7">
       <c r="A87">
         <v>2011</v>
       </c>
-      <c r="B87">
-        <v>0.6613861386138614</v>
-      </c>
-      <c r="C87">
-        <v>0.9304237824161923</v>
-      </c>
       <c r="D87" t="s">
         <v>13</v>
       </c>
       <c r="E87">
-        <v>668</v>
+        <v>1166</v>
       </c>
       <c r="F87">
-        <v>1010</v>
+        <v>0</v>
       </c>
       <c r="G87">
-        <v>1592</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88" spans="1:7">
       <c r="A88">
         <v>2012</v>
       </c>
-      <c r="B88">
-        <v>0.6505324298160697</v>
-      </c>
-      <c r="C88">
-        <v>0.9723618090452262</v>
-      </c>
       <c r="D88" t="s">
         <v>13</v>
       </c>
       <c r="E88">
-        <v>672</v>
+        <v>1287</v>
       </c>
       <c r="F88">
-        <v>1033</v>
+        <v>0</v>
       </c>
       <c r="G88">
-        <v>1705</v>
+        <v>0</v>
       </c>
     </row>
     <row r="89" spans="1:7">
       <c r="A89">
         <v>2013</v>
       </c>
-      <c r="B89">
-        <v>0.6616008105369807</v>
-      </c>
-      <c r="C89">
-        <v>0.9214076246334311</v>
-      </c>
       <c r="D89" t="s">
         <v>13</v>
       </c>
       <c r="E89">
-        <v>653</v>
+        <v>1379</v>
       </c>
       <c r="F89">
-        <v>987</v>
+        <v>0</v>
       </c>
       <c r="G89">
-        <v>1708</v>
+        <v>0</v>
       </c>
     </row>
     <row r="90" spans="1:7">
       <c r="A90">
         <v>2014</v>
       </c>
-      <c r="B90">
-        <v>0.6709677419354839</v>
-      </c>
-      <c r="C90">
-        <v>0.955503512880562</v>
-      </c>
       <c r="D90" t="s">
         <v>13</v>
       </c>
       <c r="E90">
-        <v>624</v>
+        <v>1270</v>
       </c>
       <c r="F90">
-        <v>930</v>
+        <v>0</v>
       </c>
       <c r="G90">
-        <v>1725</v>
+        <v>0</v>
       </c>
     </row>
     <row r="91" spans="1:7">
       <c r="A91">
         <v>2015</v>
       </c>
-      <c r="B91">
-        <v>0.6818181818181818</v>
-      </c>
-      <c r="C91">
-        <v>0.9739130434782609</v>
-      </c>
       <c r="D91" t="s">
         <v>13</v>
       </c>
       <c r="E91">
-        <v>615</v>
+        <v>1300</v>
       </c>
       <c r="F91">
-        <v>902</v>
+        <v>0</v>
       </c>
       <c r="G91">
-        <v>1773</v>
+        <v>0</v>
       </c>
     </row>
     <row r="92" spans="1:7">
@@ -2385,22 +2358,19 @@
         <v>2016</v>
       </c>
       <c r="B92">
-        <v>0.6379853095487933</v>
-      </c>
-      <c r="C92">
-        <v>0.9199097574732092</v>
+        <v>8.15</v>
       </c>
       <c r="D92" t="s">
         <v>13</v>
       </c>
       <c r="E92">
-        <v>608</v>
+        <v>1282</v>
       </c>
       <c r="F92">
-        <v>953</v>
+        <v>0</v>
       </c>
       <c r="G92">
-        <v>1723</v>
+        <v>0</v>
       </c>
     </row>
     <row r="93" spans="1:7">
@@ -2408,22 +2378,19 @@
         <v>2017</v>
       </c>
       <c r="B93">
-        <v>0.4535637149028078</v>
-      </c>
-      <c r="C93">
-        <v>0.9396401625072548</v>
+        <v>2.797254487856389</v>
       </c>
       <c r="D93" t="s">
         <v>13</v>
       </c>
       <c r="E93">
-        <v>420</v>
+        <v>1241</v>
       </c>
       <c r="F93">
-        <v>926</v>
+        <v>480</v>
       </c>
       <c r="G93">
-        <v>1722</v>
+        <v>1180</v>
       </c>
     </row>
     <row r="94" spans="1:7">
@@ -2431,22 +2398,22 @@
         <v>2018</v>
       </c>
       <c r="B94">
-        <v>0.2224576271186441</v>
+        <v>0.9723032069970845</v>
       </c>
       <c r="C94">
-        <v>0.8519163763066202</v>
+        <v>1.766949152542373</v>
       </c>
       <c r="D94" t="s">
         <v>13</v>
       </c>
       <c r="E94">
-        <v>210</v>
+        <v>1451</v>
       </c>
       <c r="F94">
-        <v>944</v>
+        <v>467</v>
       </c>
       <c r="G94">
-        <v>1530</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="95" spans="1:7">
@@ -2457,19 +2424,19 @@
         <v>0</v>
       </c>
       <c r="C95">
-        <v>0.9457516339869281</v>
+        <v>1.752043596730245</v>
       </c>
       <c r="D95" t="s">
         <v>13</v>
       </c>
       <c r="E95">
-        <v>0</v>
+        <v>1309</v>
       </c>
       <c r="F95">
-        <v>921</v>
+        <v>425</v>
       </c>
       <c r="G95">
-        <v>1553</v>
+        <v>1045</v>
       </c>
     </row>
     <row r="96" spans="1:7">
@@ -2480,19 +2447,19 @@
         <v>0</v>
       </c>
       <c r="C96">
-        <v>0.9253058596265293</v>
+        <v>1.873684210526316</v>
       </c>
       <c r="D96" t="s">
         <v>13</v>
       </c>
       <c r="E96">
-        <v>0</v>
+        <v>1360</v>
       </c>
       <c r="F96">
-        <v>917</v>
+        <v>387</v>
       </c>
       <c r="G96">
-        <v>1536</v>
+        <v>985</v>
       </c>
     </row>
     <row r="97" spans="1:7">
@@ -2503,19 +2470,19 @@
         <v>0</v>
       </c>
       <c r="C97">
-        <v>0.921875</v>
+        <v>1.861928934010152</v>
       </c>
       <c r="D97" t="s">
         <v>13</v>
       </c>
       <c r="E97">
-        <v>0</v>
+        <v>1263</v>
       </c>
       <c r="F97">
-        <v>910</v>
+        <v>431</v>
       </c>
       <c r="G97">
-        <v>1504</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="98" spans="1:7">
@@ -2526,19 +2493,19 @@
         <v>0</v>
       </c>
       <c r="C98">
-        <v>0.9428191489361702</v>
+        <v>1.917165668662675</v>
       </c>
       <c r="D98" t="s">
         <v>13</v>
       </c>
       <c r="E98">
-        <v>0</v>
+        <v>1315</v>
       </c>
       <c r="F98">
-        <v>874</v>
+        <v>383</v>
       </c>
       <c r="G98">
-        <v>1526</v>
+        <v>989</v>
       </c>
     </row>
     <row r="99" spans="1:7">
@@ -2549,154 +2516,121 @@
         <v>0</v>
       </c>
       <c r="C99">
-        <v>0.9823066841415465</v>
+        <v>1.845298281092012</v>
       </c>
       <c r="D99" t="s">
         <v>13</v>
       </c>
       <c r="E99">
-        <v>0</v>
+        <v>1334</v>
       </c>
       <c r="F99">
-        <v>598</v>
+        <v>384</v>
       </c>
       <c r="G99">
-        <v>1569</v>
+        <v>875</v>
       </c>
     </row>
     <row r="100" spans="1:7">
       <c r="A100">
         <v>2010</v>
       </c>
-      <c r="B100">
-        <v>1.064516129032258</v>
-      </c>
       <c r="D100" t="s">
         <v>14</v>
       </c>
       <c r="E100">
-        <v>33</v>
+        <v>354</v>
       </c>
       <c r="F100">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="G100">
-        <v>86</v>
+        <v>0</v>
       </c>
     </row>
     <row r="101" spans="1:7">
       <c r="A101">
         <v>2011</v>
       </c>
-      <c r="B101">
-        <v>0.8367346938775511</v>
-      </c>
-      <c r="C101">
-        <v>1.081395348837209</v>
-      </c>
       <c r="D101" t="s">
         <v>14</v>
       </c>
       <c r="E101">
-        <v>41</v>
+        <v>346</v>
       </c>
       <c r="F101">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="G101">
-        <v>85</v>
+        <v>0</v>
       </c>
     </row>
     <row r="102" spans="1:7">
       <c r="A102">
         <v>2012</v>
       </c>
-      <c r="B102">
-        <v>1.102040816326531</v>
-      </c>
-      <c r="C102">
-        <v>0.9411764705882353</v>
-      </c>
       <c r="D102" t="s">
         <v>14</v>
       </c>
       <c r="E102">
-        <v>54</v>
+        <v>353</v>
       </c>
       <c r="F102">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="G102">
-        <v>84</v>
+        <v>0</v>
       </c>
     </row>
     <row r="103" spans="1:7">
       <c r="A103">
         <v>2013</v>
       </c>
-      <c r="B103">
-        <v>1.081967213114754</v>
-      </c>
-      <c r="C103">
-        <v>0.9642857142857143</v>
-      </c>
       <c r="D103" t="s">
         <v>14</v>
       </c>
       <c r="E103">
-        <v>66</v>
+        <v>340</v>
       </c>
       <c r="F103">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="G103">
-        <v>91</v>
+        <v>0</v>
       </c>
     </row>
     <row r="104" spans="1:7">
       <c r="A104">
         <v>2014</v>
       </c>
-      <c r="B104">
-        <v>0.7974683544303798</v>
-      </c>
-      <c r="C104">
-        <v>0.8901098901098901</v>
-      </c>
       <c r="D104" t="s">
         <v>14</v>
       </c>
       <c r="E104">
-        <v>63</v>
+        <v>378</v>
       </c>
       <c r="F104">
-        <v>79</v>
+        <v>0</v>
       </c>
       <c r="G104">
-        <v>89</v>
+        <v>0</v>
       </c>
     </row>
     <row r="105" spans="1:7">
       <c r="A105">
         <v>2015</v>
       </c>
-      <c r="B105">
-        <v>0.8026315789473685</v>
-      </c>
-      <c r="C105">
-        <v>1.134831460674157</v>
-      </c>
       <c r="D105" t="s">
         <v>14</v>
       </c>
       <c r="E105">
-        <v>61</v>
+        <v>368</v>
       </c>
       <c r="F105">
-        <v>76</v>
+        <v>0</v>
       </c>
       <c r="G105">
-        <v>123</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106" spans="1:7">
@@ -2704,22 +2638,19 @@
         <v>2016</v>
       </c>
       <c r="B106">
-        <v>0.8767123287671232</v>
-      </c>
-      <c r="C106">
-        <v>0.9349593495934959</v>
+        <v>9.236641221374045</v>
       </c>
       <c r="D106" t="s">
         <v>14</v>
       </c>
       <c r="E106">
-        <v>64</v>
+        <v>374</v>
       </c>
       <c r="F106">
-        <v>73</v>
+        <v>0</v>
       </c>
       <c r="G106">
-        <v>123</v>
+        <v>0</v>
       </c>
     </row>
     <row r="107" spans="1:7">
@@ -2727,22 +2658,19 @@
         <v>2017</v>
       </c>
       <c r="B107">
-        <v>0.5921052631578947</v>
-      </c>
-      <c r="C107">
-        <v>0.983739837398374</v>
+        <v>3.348</v>
       </c>
       <c r="D107" t="s">
         <v>14</v>
       </c>
       <c r="E107">
-        <v>45</v>
+        <v>394</v>
       </c>
       <c r="F107">
-        <v>76</v>
+        <v>131</v>
       </c>
       <c r="G107">
-        <v>131</v>
+        <v>376</v>
       </c>
     </row>
     <row r="108" spans="1:7">
@@ -2750,22 +2678,22 @@
         <v>2018</v>
       </c>
       <c r="B108">
-        <v>0.2926829268292683</v>
+        <v>1.239193083573487</v>
       </c>
       <c r="C108">
-        <v>0.9007633587786259</v>
+        <v>1.75531914893617</v>
       </c>
       <c r="D108" t="s">
         <v>14</v>
       </c>
       <c r="E108">
-        <v>24</v>
+        <v>443</v>
       </c>
       <c r="F108">
-        <v>82</v>
+        <v>119</v>
       </c>
       <c r="G108">
-        <v>135</v>
+        <v>336</v>
       </c>
     </row>
     <row r="109" spans="1:7">
@@ -2776,19 +2704,19 @@
         <v>0</v>
       </c>
       <c r="C109">
-        <v>0.9925925925925926</v>
+        <v>1.636904761904762</v>
       </c>
       <c r="D109" t="s">
         <v>14</v>
       </c>
       <c r="E109">
-        <v>0</v>
+        <v>359</v>
       </c>
       <c r="F109">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="G109">
-        <v>135</v>
+        <v>288</v>
       </c>
     </row>
     <row r="110" spans="1:7">
@@ -2799,19 +2727,19 @@
         <v>0</v>
       </c>
       <c r="C110">
-        <v>0.9555555555555556</v>
+        <v>1.958333333333333</v>
       </c>
       <c r="D110" t="s">
         <v>14</v>
       </c>
       <c r="E110">
-        <v>0</v>
+        <v>407</v>
       </c>
       <c r="F110">
-        <v>96</v>
+        <v>117</v>
       </c>
       <c r="G110">
-        <v>151</v>
+        <v>274</v>
       </c>
     </row>
     <row r="111" spans="1:7">
@@ -2822,19 +2750,19 @@
         <v>0</v>
       </c>
       <c r="C111">
-        <v>1.006622516556291</v>
+        <v>2.029197080291971</v>
       </c>
       <c r="D111" t="s">
         <v>14</v>
       </c>
       <c r="E111">
-        <v>0</v>
+        <v>373</v>
       </c>
       <c r="F111">
-        <v>110</v>
+        <v>144</v>
       </c>
       <c r="G111">
-        <v>162</v>
+        <v>327</v>
       </c>
     </row>
     <row r="112" spans="1:7">
@@ -2845,19 +2773,19 @@
         <v>0</v>
       </c>
       <c r="C112">
-        <v>0.9814814814814815</v>
+        <v>1.819571865443425</v>
       </c>
       <c r="D112" t="s">
         <v>14</v>
       </c>
       <c r="E112">
-        <v>0</v>
+        <v>407</v>
       </c>
       <c r="F112">
-        <v>110</v>
+        <v>141</v>
       </c>
       <c r="G112">
-        <v>176</v>
+        <v>329</v>
       </c>
     </row>
     <row r="113" spans="1:7">
@@ -2868,19 +2796,19 @@
         <v>0</v>
       </c>
       <c r="C113">
-        <v>1.022727272727273</v>
+        <v>1.838905775075988</v>
       </c>
       <c r="D113" t="s">
         <v>14</v>
       </c>
       <c r="E113">
-        <v>0</v>
+        <v>430</v>
       </c>
       <c r="F113">
-        <v>81</v>
+        <v>128</v>
       </c>
       <c r="G113">
-        <v>199</v>
+        <v>303</v>
       </c>
     </row>
     <row r="114" spans="1:7">
@@ -2888,19 +2816,19 @@
         <v>2010</v>
       </c>
       <c r="B114">
-        <v>0.75</v>
+        <v>0.9270678290452903</v>
       </c>
       <c r="D114" t="s">
         <v>15</v>
       </c>
       <c r="E114">
-        <v>6</v>
+        <v>514</v>
       </c>
       <c r="F114">
-        <v>8</v>
+        <v>2258</v>
       </c>
       <c r="G114">
-        <v>20</v>
+        <v>10960</v>
       </c>
     </row>
     <row r="115" spans="1:7">
@@ -2908,22 +2836,22 @@
         <v>2011</v>
       </c>
       <c r="B115">
-        <v>0.4615384615384616</v>
+        <v>0.6391826236067448</v>
       </c>
       <c r="C115">
-        <v>1.1</v>
+        <v>0.9498175182481752</v>
       </c>
       <c r="D115" t="s">
         <v>15</v>
       </c>
       <c r="E115">
-        <v>6</v>
+        <v>1358</v>
       </c>
       <c r="F115">
-        <v>13</v>
+        <v>2445</v>
       </c>
       <c r="G115">
-        <v>19</v>
+        <v>11497</v>
       </c>
     </row>
     <row r="116" spans="1:7">
@@ -2931,22 +2859,22 @@
         <v>2012</v>
       </c>
       <c r="B116">
-        <v>0.3636363636363636</v>
+        <v>0.6308258960192662</v>
       </c>
       <c r="C116">
-        <v>1.105263157894737</v>
+        <v>0.9038009915630164</v>
       </c>
       <c r="D116" t="s">
         <v>15</v>
       </c>
       <c r="E116">
-        <v>4</v>
+        <v>1442</v>
       </c>
       <c r="F116">
-        <v>11</v>
+        <v>2295</v>
       </c>
       <c r="G116">
-        <v>22</v>
+        <v>11244</v>
       </c>
     </row>
     <row r="117" spans="1:7">
@@ -2954,22 +2882,22 @@
         <v>2013</v>
       </c>
       <c r="B117">
-        <v>0.2857142857142857</v>
+        <v>0.665936313175577</v>
       </c>
       <c r="C117">
-        <v>0.6818181818181818</v>
+        <v>0.9447705442902882</v>
       </c>
       <c r="D117" t="s">
         <v>15</v>
       </c>
       <c r="E117">
-        <v>4</v>
+        <v>1501</v>
       </c>
       <c r="F117">
-        <v>14</v>
+        <v>2319</v>
       </c>
       <c r="G117">
-        <v>17</v>
+        <v>11441</v>
       </c>
     </row>
     <row r="118" spans="1:7">
@@ -2977,22 +2905,22 @@
         <v>2014</v>
       </c>
       <c r="B118">
-        <v>0.4</v>
+        <v>0.6342395297575312</v>
       </c>
       <c r="C118">
-        <v>1</v>
+        <v>0.9562101214928765</v>
       </c>
       <c r="D118" t="s">
         <v>15</v>
       </c>
       <c r="E118">
-        <v>6</v>
+        <v>1462</v>
       </c>
       <c r="F118">
-        <v>15</v>
+        <v>2232</v>
       </c>
       <c r="G118">
-        <v>19</v>
+        <v>11710</v>
       </c>
     </row>
     <row r="119" spans="1:7">
@@ -3000,22 +2928,22 @@
         <v>2015</v>
       </c>
       <c r="B119">
-        <v>0.5625</v>
+        <v>0.6402718274486631</v>
       </c>
       <c r="C119">
-        <v>0.7894736842105263</v>
+        <v>0.9151152860802733</v>
       </c>
       <c r="D119" t="s">
         <v>15</v>
       </c>
       <c r="E119">
-        <v>9</v>
+        <v>1465</v>
       </c>
       <c r="F119">
-        <v>16</v>
+        <v>2254</v>
       </c>
       <c r="G119">
-        <v>20</v>
+        <v>11505</v>
       </c>
     </row>
     <row r="120" spans="1:7">
@@ -3023,22 +2951,22 @@
         <v>2016</v>
       </c>
       <c r="B120">
-        <v>0.6</v>
+        <v>0.6307023895727734</v>
       </c>
       <c r="C120">
-        <v>0.8</v>
+        <v>0.937070838765754</v>
       </c>
       <c r="D120" t="s">
         <v>15</v>
       </c>
       <c r="E120">
-        <v>12</v>
+        <v>1489</v>
       </c>
       <c r="F120">
-        <v>20</v>
+        <v>2283</v>
       </c>
       <c r="G120">
-        <v>18</v>
+        <v>11575</v>
       </c>
     </row>
     <row r="121" spans="1:7">
@@ -3046,22 +2974,22 @@
         <v>2017</v>
       </c>
       <c r="B121">
-        <v>0.3333333333333333</v>
+        <v>0.4354094579008074</v>
       </c>
       <c r="C121">
-        <v>1</v>
+        <v>0.9042764578833693</v>
       </c>
       <c r="D121" t="s">
         <v>15</v>
       </c>
       <c r="E121">
-        <v>9</v>
+        <v>1406</v>
       </c>
       <c r="F121">
-        <v>27</v>
+        <v>2368</v>
       </c>
       <c r="G121">
-        <v>25</v>
+        <v>11429</v>
       </c>
     </row>
     <row r="122" spans="1:7">
@@ -3069,22 +2997,22 @@
         <v>2018</v>
       </c>
       <c r="B122">
-        <v>0.1785714285714286</v>
+        <v>0.2195331519404267</v>
       </c>
       <c r="C122">
-        <v>0.88</v>
+        <v>0.9056785370548605</v>
       </c>
       <c r="D122" t="s">
         <v>15</v>
       </c>
       <c r="E122">
-        <v>5</v>
+        <v>1578</v>
       </c>
       <c r="F122">
-        <v>28</v>
+        <v>2285</v>
       </c>
       <c r="G122">
-        <v>34</v>
+        <v>11058</v>
       </c>
     </row>
     <row r="123" spans="1:7">
@@ -3095,19 +3023,19 @@
         <v>0</v>
       </c>
       <c r="C123">
-        <v>0.8235294117647058</v>
+        <v>0.9177066377283415</v>
       </c>
       <c r="D123" t="s">
         <v>15</v>
       </c>
       <c r="E123">
-        <v>0</v>
+        <v>1469</v>
       </c>
       <c r="F123">
-        <v>22</v>
+        <v>2330</v>
       </c>
       <c r="G123">
-        <v>33</v>
+        <v>11009</v>
       </c>
     </row>
     <row r="124" spans="1:7">
@@ -3118,19 +3046,19 @@
         <v>0</v>
       </c>
       <c r="C124">
-        <v>0.9090909090909091</v>
+        <v>0.9332364429103461</v>
       </c>
       <c r="D124" t="s">
         <v>15</v>
       </c>
       <c r="E124">
-        <v>0</v>
+        <v>1512</v>
       </c>
       <c r="F124">
-        <v>12</v>
+        <v>2280</v>
       </c>
       <c r="G124">
-        <v>31</v>
+        <v>11042</v>
       </c>
     </row>
     <row r="125" spans="1:7">
@@ -3141,19 +3069,19 @@
         <v>0</v>
       </c>
       <c r="C125">
-        <v>1.032258064516129</v>
+        <v>0.9386886433617099</v>
       </c>
       <c r="D125" t="s">
         <v>15</v>
       </c>
       <c r="E125">
-        <v>0</v>
+        <v>1335</v>
       </c>
       <c r="F125">
-        <v>19</v>
+        <v>2240</v>
       </c>
       <c r="G125">
-        <v>32</v>
+        <v>11270</v>
       </c>
     </row>
     <row r="126" spans="1:7">
@@ -3164,19 +3092,19 @@
         <v>0</v>
       </c>
       <c r="C126">
-        <v>0.875</v>
+        <v>0.9204968944099379</v>
       </c>
       <c r="D126" t="s">
         <v>15</v>
       </c>
       <c r="E126">
-        <v>0</v>
+        <v>1487</v>
       </c>
       <c r="F126">
-        <v>24</v>
+        <v>2143</v>
       </c>
       <c r="G126">
-        <v>37</v>
+        <v>11030</v>
       </c>
     </row>
     <row r="127" spans="1:7">
@@ -3187,19 +3115,19 @@
         <v>0</v>
       </c>
       <c r="C127">
-        <v>0.972972972972973</v>
+        <v>0.9485040797824116</v>
       </c>
       <c r="D127" t="s">
         <v>15</v>
       </c>
       <c r="E127">
-        <v>0</v>
+        <v>1533</v>
       </c>
       <c r="F127">
-        <v>21</v>
+        <v>2084</v>
       </c>
       <c r="G127">
-        <v>39</v>
+        <v>11013</v>
       </c>
     </row>
     <row r="128" spans="1:7">
@@ -3207,19 +3135,19 @@
         <v>2010</v>
       </c>
       <c r="B128">
-        <v>0.9230769230769231</v>
+        <v>1.214076246334311</v>
       </c>
       <c r="D128" t="s">
         <v>16</v>
       </c>
       <c r="E128">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="F128">
-        <v>26</v>
+        <v>170</v>
       </c>
       <c r="G128">
-        <v>68</v>
+        <v>865</v>
       </c>
     </row>
     <row r="129" spans="1:7">
@@ -3227,22 +3155,22 @@
         <v>2011</v>
       </c>
       <c r="B129">
-        <v>0.6857142857142857</v>
+        <v>0.8426966292134831</v>
       </c>
       <c r="C129">
-        <v>0.8970588235294118</v>
+        <v>1.064739884393064</v>
       </c>
       <c r="D129" t="s">
         <v>16</v>
       </c>
       <c r="E129">
-        <v>24</v>
+        <v>121</v>
       </c>
       <c r="F129">
-        <v>35</v>
+        <v>171</v>
       </c>
       <c r="G129">
-        <v>69</v>
+        <v>971</v>
       </c>
     </row>
     <row r="130" spans="1:7">
@@ -3250,22 +3178,22 @@
         <v>2012</v>
       </c>
       <c r="B130">
-        <v>0.7209302325581395</v>
+        <v>0.7888513513513513</v>
       </c>
       <c r="C130">
-        <v>0.8840579710144928</v>
+        <v>0.9258496395468589</v>
       </c>
       <c r="D130" t="s">
         <v>16</v>
       </c>
       <c r="E130">
-        <v>31</v>
+        <v>124</v>
       </c>
       <c r="F130">
-        <v>43</v>
+        <v>193</v>
       </c>
       <c r="G130">
-        <v>57</v>
+        <v>968</v>
       </c>
     </row>
     <row r="131" spans="1:7">
@@ -3273,22 +3201,22 @@
         <v>2013</v>
       </c>
       <c r="B131">
-        <v>0.6041666666666666</v>
+        <v>0.7432216905901117</v>
       </c>
       <c r="C131">
-        <v>0.9649122807017544</v>
+        <v>0.987603305785124</v>
       </c>
       <c r="D131" t="s">
         <v>16</v>
       </c>
       <c r="E131">
-        <v>29</v>
+        <v>136</v>
       </c>
       <c r="F131">
-        <v>48</v>
+        <v>228</v>
       </c>
       <c r="G131">
-        <v>71</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="132" spans="1:7">
@@ -3296,22 +3224,22 @@
         <v>2014</v>
       </c>
       <c r="B132">
-        <v>0.5245901639344263</v>
+        <v>0.6642011834319527</v>
       </c>
       <c r="C132">
-        <v>0.9154929577464789</v>
+        <v>0.9284351145038168</v>
       </c>
       <c r="D132" t="s">
         <v>16</v>
       </c>
       <c r="E132">
-        <v>32</v>
+        <v>136</v>
       </c>
       <c r="F132">
-        <v>61</v>
+        <v>206</v>
       </c>
       <c r="G132">
-        <v>72</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="133" spans="1:7">
@@ -3319,22 +3247,22 @@
         <v>2015</v>
       </c>
       <c r="B133">
-        <v>0.6428571428571429</v>
+        <v>0.7443946188340808</v>
       </c>
       <c r="C133">
-        <v>1.027777777777778</v>
+        <v>0.9808245445829339</v>
       </c>
       <c r="D133" t="s">
         <v>16</v>
       </c>
       <c r="E133">
-        <v>36</v>
+        <v>123</v>
       </c>
       <c r="F133">
-        <v>56</v>
+        <v>242</v>
       </c>
       <c r="G133">
-        <v>90</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="134" spans="1:7">
@@ -3342,22 +3270,22 @@
         <v>2016</v>
       </c>
       <c r="B134">
-        <v>0.5443037974683544</v>
+        <v>0.818830242510699</v>
       </c>
       <c r="C134">
-        <v>0.8666666666666667</v>
+        <v>1.019264448336252</v>
       </c>
       <c r="D134" t="s">
         <v>16</v>
       </c>
       <c r="E134">
-        <v>43</v>
+        <v>141</v>
       </c>
       <c r="F134">
-        <v>79</v>
+        <v>221</v>
       </c>
       <c r="G134">
-        <v>88</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="135" spans="1:7">
@@ -3365,22 +3293,22 @@
         <v>2017</v>
       </c>
       <c r="B135">
-        <v>0.3505154639175257</v>
+        <v>0.5454545454545454</v>
       </c>
       <c r="C135">
-        <v>1.045454545454545</v>
+        <v>0.9003215434083601</v>
       </c>
       <c r="D135" t="s">
         <v>16</v>
       </c>
       <c r="E135">
-        <v>34</v>
+        <v>150</v>
       </c>
       <c r="F135">
-        <v>97</v>
+        <v>238</v>
       </c>
       <c r="G135">
-        <v>121</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="136" spans="1:7">
@@ -3388,22 +3316,22 @@
         <v>2018</v>
       </c>
       <c r="B136">
-        <v>0.1574074074074074</v>
+        <v>0.2723970944309927</v>
       </c>
       <c r="C136">
-        <v>0.8016528925619835</v>
+        <v>0.9478476821192053</v>
       </c>
       <c r="D136" t="s">
         <v>16</v>
       </c>
       <c r="E136">
-        <v>17</v>
+        <v>159</v>
       </c>
       <c r="F136">
-        <v>108</v>
+        <v>333</v>
       </c>
       <c r="G136">
-        <v>131</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="137" spans="1:7">
@@ -3414,19 +3342,19 @@
         <v>0</v>
       </c>
       <c r="C137">
-        <v>0.9618320610687023</v>
+        <v>0.9044730856709629</v>
       </c>
       <c r="D137" t="s">
         <v>16</v>
       </c>
       <c r="E137">
-        <v>0</v>
+        <v>158</v>
       </c>
       <c r="F137">
-        <v>100</v>
+        <v>255</v>
       </c>
       <c r="G137">
-        <v>140</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="138" spans="1:7">
@@ -3437,19 +3365,19 @@
         <v>0</v>
       </c>
       <c r="C138">
-        <v>0.8214285714285714</v>
+        <v>0.9558139534883721</v>
       </c>
       <c r="D138" t="s">
         <v>16</v>
       </c>
       <c r="E138">
-        <v>0</v>
+        <v>149</v>
       </c>
       <c r="F138">
-        <v>97</v>
+        <v>302</v>
       </c>
       <c r="G138">
-        <v>138</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="139" spans="1:7">
@@ -3460,19 +3388,19 @@
         <v>0</v>
       </c>
       <c r="C139">
-        <v>0.9492753623188406</v>
+        <v>0.9487734487734488</v>
       </c>
       <c r="D139" t="s">
         <v>16</v>
       </c>
       <c r="E139">
-        <v>0</v>
+        <v>142</v>
       </c>
       <c r="F139">
-        <v>98</v>
+        <v>354</v>
       </c>
       <c r="G139">
-        <v>159</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="140" spans="1:7">
@@ -3483,19 +3411,19 @@
         <v>0</v>
       </c>
       <c r="C140">
-        <v>0.89937106918239</v>
+        <v>0.9685658153241651</v>
       </c>
       <c r="D140" t="s">
         <v>16</v>
       </c>
       <c r="E140">
-        <v>0</v>
+        <v>207</v>
       </c>
       <c r="F140">
-        <v>104</v>
+        <v>355</v>
       </c>
       <c r="G140">
-        <v>154</v>
+        <v>1627</v>
       </c>
     </row>
     <row r="141" spans="1:7">
@@ -3506,19 +3434,657 @@
         <v>0</v>
       </c>
       <c r="C141">
-        <v>1.038961038961039</v>
+        <v>0.9551321450522434</v>
       </c>
       <c r="D141" t="s">
         <v>16</v>
       </c>
       <c r="E141">
-        <v>0</v>
+        <v>225</v>
       </c>
       <c r="F141">
-        <v>67</v>
+        <v>361</v>
       </c>
       <c r="G141">
-        <v>182</v>
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7">
+      <c r="A142">
+        <v>2010</v>
+      </c>
+      <c r="B142">
+        <v>1.166666666666667</v>
+      </c>
+      <c r="D142" t="s">
+        <v>17</v>
+      </c>
+      <c r="E142">
+        <v>18</v>
+      </c>
+      <c r="F142">
+        <v>74</v>
+      </c>
+      <c r="G142">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7">
+      <c r="A143">
+        <v>2011</v>
+      </c>
+      <c r="B143">
+        <v>0.8354430379746836</v>
+      </c>
+      <c r="C143">
+        <v>1.114982578397212</v>
+      </c>
+      <c r="D143" t="s">
+        <v>17</v>
+      </c>
+      <c r="E143">
+        <v>49</v>
+      </c>
+      <c r="F143">
+        <v>40</v>
+      </c>
+      <c r="G143">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7">
+      <c r="A144">
+        <v>2012</v>
+      </c>
+      <c r="B144">
+        <v>0.8581081081081081</v>
+      </c>
+      <c r="C144">
+        <v>0.8553054662379421</v>
+      </c>
+      <c r="D144" t="s">
+        <v>17</v>
+      </c>
+      <c r="E144">
+        <v>39</v>
+      </c>
+      <c r="F144">
+        <v>44</v>
+      </c>
+      <c r="G144">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7">
+      <c r="A145">
+        <v>2013</v>
+      </c>
+      <c r="B145">
+        <v>0.7911392405063291</v>
+      </c>
+      <c r="C145">
+        <v>0.959409594095941</v>
+      </c>
+      <c r="D145" t="s">
+        <v>17</v>
+      </c>
+      <c r="E145">
+        <v>53</v>
+      </c>
+      <c r="F145">
+        <v>64</v>
+      </c>
+      <c r="G145">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7">
+      <c r="A146">
+        <v>2014</v>
+      </c>
+      <c r="B146">
+        <v>0.7076023391812866</v>
+      </c>
+      <c r="C146">
+        <v>0.955719557195572</v>
+      </c>
+      <c r="D146" t="s">
+        <v>17</v>
+      </c>
+      <c r="E146">
+        <v>41</v>
+      </c>
+      <c r="F146">
+        <v>50</v>
+      </c>
+      <c r="G146">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7">
+      <c r="A147">
+        <v>2015</v>
+      </c>
+      <c r="B147">
+        <v>0.676923076923077</v>
+      </c>
+      <c r="C147">
+        <v>0.9328358208955224</v>
+      </c>
+      <c r="D147" t="s">
+        <v>17</v>
+      </c>
+      <c r="E147">
+        <v>41</v>
+      </c>
+      <c r="F147">
+        <v>57</v>
+      </c>
+      <c r="G147">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7">
+      <c r="A148">
+        <v>2016</v>
+      </c>
+      <c r="B148">
+        <v>0.5234375</v>
+      </c>
+      <c r="C148">
+        <v>0.8082706766917294</v>
+      </c>
+      <c r="D148" t="s">
+        <v>17</v>
+      </c>
+      <c r="E148">
+        <v>41</v>
+      </c>
+      <c r="F148">
+        <v>88</v>
+      </c>
+      <c r="G148">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7">
+      <c r="A149">
+        <v>2017</v>
+      </c>
+      <c r="B149">
+        <v>0.3121019108280255</v>
+      </c>
+      <c r="C149">
+        <v>1.072519083969466</v>
+      </c>
+      <c r="D149" t="s">
+        <v>17</v>
+      </c>
+      <c r="E149">
+        <v>51</v>
+      </c>
+      <c r="F149">
+        <v>111</v>
+      </c>
+      <c r="G149">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7">
+      <c r="A150">
+        <v>2018</v>
+      </c>
+      <c r="B150">
+        <v>0.1522388059701492</v>
+      </c>
+      <c r="C150">
+        <v>0.9442815249266863</v>
+      </c>
+      <c r="D150" t="s">
+        <v>17</v>
+      </c>
+      <c r="E150">
+        <v>40</v>
+      </c>
+      <c r="F150">
+        <v>115</v>
+      </c>
+      <c r="G150">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7">
+      <c r="A151">
+        <v>2019</v>
+      </c>
+      <c r="B151">
+        <v>0</v>
+      </c>
+      <c r="C151">
+        <v>0.8261964735516373</v>
+      </c>
+      <c r="D151" t="s">
+        <v>17</v>
+      </c>
+      <c r="E151">
+        <v>36</v>
+      </c>
+      <c r="F151">
+        <v>109</v>
+      </c>
+      <c r="G151">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7">
+      <c r="A152">
+        <v>2020</v>
+      </c>
+      <c r="B152">
+        <v>0</v>
+      </c>
+      <c r="C152">
+        <v>0.9226932668329177</v>
+      </c>
+      <c r="D152" t="s">
+        <v>17</v>
+      </c>
+      <c r="E152">
+        <v>49</v>
+      </c>
+      <c r="F152">
+        <v>106</v>
+      </c>
+      <c r="G152">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7">
+      <c r="A153">
+        <v>2021</v>
+      </c>
+      <c r="B153">
+        <v>0</v>
+      </c>
+      <c r="C153">
+        <v>0.8618266978922716</v>
+      </c>
+      <c r="D153" t="s">
+        <v>17</v>
+      </c>
+      <c r="E153">
+        <v>36</v>
+      </c>
+      <c r="F153">
+        <v>111</v>
+      </c>
+      <c r="G153">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7">
+      <c r="A154">
+        <v>2022</v>
+      </c>
+      <c r="B154">
+        <v>0</v>
+      </c>
+      <c r="C154">
+        <v>0.8848758465011287</v>
+      </c>
+      <c r="D154" t="s">
+        <v>17</v>
+      </c>
+      <c r="E154">
+        <v>47</v>
+      </c>
+      <c r="F154">
+        <v>127</v>
+      </c>
+      <c r="G154">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7">
+      <c r="A155">
+        <v>2023</v>
+      </c>
+      <c r="B155">
+        <v>0</v>
+      </c>
+      <c r="C155">
+        <v>0.902542372881356</v>
+      </c>
+      <c r="D155" t="s">
+        <v>17</v>
+      </c>
+      <c r="E155">
+        <v>51</v>
+      </c>
+      <c r="F155">
+        <v>109</v>
+      </c>
+      <c r="G155">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7">
+      <c r="A156">
+        <v>2010</v>
+      </c>
+      <c r="B156">
+        <v>1.252525252525253</v>
+      </c>
+      <c r="D156" t="s">
+        <v>18</v>
+      </c>
+      <c r="E156">
+        <v>33</v>
+      </c>
+      <c r="F156">
+        <v>131</v>
+      </c>
+      <c r="G156">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7">
+      <c r="A157">
+        <v>2011</v>
+      </c>
+      <c r="B157">
+        <v>0.9029345372460497</v>
+      </c>
+      <c r="C157">
+        <v>0.9299552906110283</v>
+      </c>
+      <c r="D157" t="s">
+        <v>18</v>
+      </c>
+      <c r="E157">
+        <v>77</v>
+      </c>
+      <c r="F157">
+        <v>166</v>
+      </c>
+      <c r="G157">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7">
+      <c r="A158">
+        <v>2012</v>
+      </c>
+      <c r="B158">
+        <v>0.9683544303797469</v>
+      </c>
+      <c r="C158">
+        <v>0.8849929873772791</v>
+      </c>
+      <c r="D158" t="s">
+        <v>18</v>
+      </c>
+      <c r="E158">
+        <v>109</v>
+      </c>
+      <c r="F158">
+        <v>146</v>
+      </c>
+      <c r="G158">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7">
+      <c r="A159">
+        <v>2013</v>
+      </c>
+      <c r="B159">
+        <v>0.9041353383458647</v>
+      </c>
+      <c r="C159">
+        <v>1.026946107784431</v>
+      </c>
+      <c r="D159" t="s">
+        <v>18</v>
+      </c>
+      <c r="E159">
+        <v>97</v>
+      </c>
+      <c r="F159">
+        <v>162</v>
+      </c>
+      <c r="G159">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7">
+      <c r="A160">
+        <v>2014</v>
+      </c>
+      <c r="B160">
+        <v>0.8174726989079563</v>
+      </c>
+      <c r="C160">
+        <v>1.029294274300932</v>
+      </c>
+      <c r="D160" t="s">
+        <v>18</v>
+      </c>
+      <c r="E160">
+        <v>109</v>
+      </c>
+      <c r="F160">
+        <v>224</v>
+      </c>
+      <c r="G160">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7">
+      <c r="A161">
+        <v>2015</v>
+      </c>
+      <c r="B161">
+        <v>0.7434895833333334</v>
+      </c>
+      <c r="C161">
+        <v>0.9403153153153153</v>
+      </c>
+      <c r="D161" t="s">
+        <v>18</v>
+      </c>
+      <c r="E161">
+        <v>122</v>
+      </c>
+      <c r="F161">
+        <v>255</v>
+      </c>
+      <c r="G161">
+        <v>968</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7">
+      <c r="A162">
+        <v>2016</v>
+      </c>
+      <c r="B162">
+        <v>0.7244546498277842</v>
+      </c>
+      <c r="C162">
+        <v>0.9328512396694215</v>
+      </c>
+      <c r="D162" t="s">
+        <v>18</v>
+      </c>
+      <c r="E162">
+        <v>115</v>
+      </c>
+      <c r="F162">
+        <v>289</v>
+      </c>
+      <c r="G162">
+        <v>1077</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7">
+      <c r="A163">
+        <v>2017</v>
+      </c>
+      <c r="B163">
+        <v>0.4591194968553459</v>
+      </c>
+      <c r="C163">
+        <v>0.9795728876508821</v>
+      </c>
+      <c r="D163" t="s">
+        <v>18</v>
+      </c>
+      <c r="E163">
+        <v>135</v>
+      </c>
+      <c r="F163">
+        <v>327</v>
+      </c>
+      <c r="G163">
+        <v>1247</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7">
+      <c r="A164">
+        <v>2018</v>
+      </c>
+      <c r="B164">
+        <v>0.2112950340798442</v>
+      </c>
+      <c r="C164">
+        <v>0.917401764234162</v>
+      </c>
+      <c r="D164" t="s">
+        <v>18</v>
+      </c>
+      <c r="E164">
+        <v>150</v>
+      </c>
+      <c r="F164">
+        <v>338</v>
+      </c>
+      <c r="G164">
+        <v>1332</v>
+      </c>
+    </row>
+    <row r="165" spans="1:7">
+      <c r="A165">
+        <v>2019</v>
+      </c>
+      <c r="B165">
+        <v>0</v>
+      </c>
+      <c r="C165">
+        <v>0.9459459459459459</v>
+      </c>
+      <c r="D165" t="s">
+        <v>18</v>
+      </c>
+      <c r="E165">
+        <v>174</v>
+      </c>
+      <c r="F165">
+        <v>362</v>
+      </c>
+      <c r="G165">
+        <v>1448</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7">
+      <c r="A166">
+        <v>2020</v>
+      </c>
+      <c r="B166">
+        <v>0</v>
+      </c>
+      <c r="C166">
+        <v>0.9060773480662984</v>
+      </c>
+      <c r="D166" t="s">
+        <v>18</v>
+      </c>
+      <c r="E166">
+        <v>157</v>
+      </c>
+      <c r="F166">
+        <v>413</v>
+      </c>
+      <c r="G166">
+        <v>1568</v>
+      </c>
+    </row>
+    <row r="167" spans="1:7">
+      <c r="A167">
+        <v>2021</v>
+      </c>
+      <c r="B167">
+        <v>0</v>
+      </c>
+      <c r="C167">
+        <v>0.9572704081632653</v>
+      </c>
+      <c r="D167" t="s">
+        <v>18</v>
+      </c>
+      <c r="E167">
+        <v>193</v>
+      </c>
+      <c r="F167">
+        <v>460</v>
+      </c>
+      <c r="G167">
+        <v>1768</v>
+      </c>
+    </row>
+    <row r="168" spans="1:7">
+      <c r="A168">
+        <v>2022</v>
+      </c>
+      <c r="B168">
+        <v>0</v>
+      </c>
+      <c r="C168">
+        <v>0.9010180995475113</v>
+      </c>
+      <c r="D168" t="s">
+        <v>18</v>
+      </c>
+      <c r="E168">
+        <v>221</v>
+      </c>
+      <c r="F168">
+        <v>355</v>
+      </c>
+      <c r="G168">
+        <v>1727</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7">
+      <c r="A169">
+        <v>2023</v>
+      </c>
+      <c r="B169">
+        <v>0</v>
+      </c>
+      <c r="C169">
+        <v>0.9270411117544876</v>
+      </c>
+      <c r="D169" t="s">
+        <v>18</v>
+      </c>
+      <c r="E169">
+        <v>217</v>
+      </c>
+      <c r="F169">
+        <v>418</v>
+      </c>
+      <c r="G169">
+        <v>1802</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added a new Multipule imputation code to create a Excel file to graph off of as well as added the neccesary extended variables to GSS trim file, finaly PCR values seem to be off to be fixed asap
</commit_message>
<xml_diff>
--- a/graphs/PCR_Retention_National.xlsx
+++ b/graphs/PCR_Retention_National.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="20">
   <si>
     <t>year</t>
   </si>
@@ -55,12 +55,6 @@
     <t>Women Doctor</t>
   </si>
   <si>
-    <t>Men Masters</t>
-  </si>
-  <si>
-    <t>Women Masters</t>
-  </si>
-  <si>
     <t>White</t>
   </si>
   <si>
@@ -71,6 +65,15 @@
   </si>
   <si>
     <t>Hispanic</t>
+  </si>
+  <si>
+    <t>Black Women</t>
+  </si>
+  <si>
+    <t>Asian Women</t>
+  </si>
+  <si>
+    <t>Hispanic Women</t>
   </si>
 </sst>
 </file>
@@ -428,7 +431,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G169"/>
+  <dimension ref="A1:G183"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -2255,102 +2258,135 @@
       <c r="A86">
         <v>2010</v>
       </c>
+      <c r="B86">
+        <v>0.9270678290452903</v>
+      </c>
       <c r="D86" t="s">
         <v>13</v>
       </c>
       <c r="E86">
-        <v>1218</v>
+        <v>514</v>
       </c>
       <c r="F86">
-        <v>0</v>
+        <v>2258</v>
       </c>
       <c r="G86">
-        <v>0</v>
+        <v>10960</v>
       </c>
     </row>
     <row r="87" spans="1:7">
       <c r="A87">
         <v>2011</v>
       </c>
+      <c r="B87">
+        <v>0.6391826236067448</v>
+      </c>
+      <c r="C87">
+        <v>0.9498175182481752</v>
+      </c>
       <c r="D87" t="s">
         <v>13</v>
       </c>
       <c r="E87">
-        <v>1166</v>
+        <v>1358</v>
       </c>
       <c r="F87">
-        <v>0</v>
+        <v>2445</v>
       </c>
       <c r="G87">
-        <v>0</v>
+        <v>11497</v>
       </c>
     </row>
     <row r="88" spans="1:7">
       <c r="A88">
         <v>2012</v>
       </c>
+      <c r="B88">
+        <v>0.6308258960192662</v>
+      </c>
+      <c r="C88">
+        <v>0.9038009915630164</v>
+      </c>
       <c r="D88" t="s">
         <v>13</v>
       </c>
       <c r="E88">
-        <v>1287</v>
+        <v>1442</v>
       </c>
       <c r="F88">
-        <v>0</v>
+        <v>2295</v>
       </c>
       <c r="G88">
-        <v>0</v>
+        <v>11244</v>
       </c>
     </row>
     <row r="89" spans="1:7">
       <c r="A89">
         <v>2013</v>
       </c>
+      <c r="B89">
+        <v>0.665936313175577</v>
+      </c>
+      <c r="C89">
+        <v>0.9447705442902882</v>
+      </c>
       <c r="D89" t="s">
         <v>13</v>
       </c>
       <c r="E89">
-        <v>1379</v>
+        <v>1501</v>
       </c>
       <c r="F89">
-        <v>0</v>
+        <v>2319</v>
       </c>
       <c r="G89">
-        <v>0</v>
+        <v>11441</v>
       </c>
     </row>
     <row r="90" spans="1:7">
       <c r="A90">
         <v>2014</v>
       </c>
+      <c r="B90">
+        <v>0.6342395297575312</v>
+      </c>
+      <c r="C90">
+        <v>0.9562101214928765</v>
+      </c>
       <c r="D90" t="s">
         <v>13</v>
       </c>
       <c r="E90">
-        <v>1270</v>
+        <v>1462</v>
       </c>
       <c r="F90">
-        <v>0</v>
+        <v>2232</v>
       </c>
       <c r="G90">
-        <v>0</v>
+        <v>11710</v>
       </c>
     </row>
     <row r="91" spans="1:7">
       <c r="A91">
         <v>2015</v>
       </c>
+      <c r="B91">
+        <v>0.6402718274486631</v>
+      </c>
+      <c r="C91">
+        <v>0.9151152860802733</v>
+      </c>
       <c r="D91" t="s">
         <v>13</v>
       </c>
       <c r="E91">
-        <v>1300</v>
+        <v>1465</v>
       </c>
       <c r="F91">
-        <v>0</v>
+        <v>2254</v>
       </c>
       <c r="G91">
-        <v>0</v>
+        <v>11505</v>
       </c>
     </row>
     <row r="92" spans="1:7">
@@ -2358,19 +2394,22 @@
         <v>2016</v>
       </c>
       <c r="B92">
-        <v>8.15</v>
+        <v>0.6307023895727734</v>
+      </c>
+      <c r="C92">
+        <v>0.937070838765754</v>
       </c>
       <c r="D92" t="s">
         <v>13</v>
       </c>
       <c r="E92">
-        <v>1282</v>
+        <v>1489</v>
       </c>
       <c r="F92">
-        <v>0</v>
+        <v>2283</v>
       </c>
       <c r="G92">
-        <v>0</v>
+        <v>11575</v>
       </c>
     </row>
     <row r="93" spans="1:7">
@@ -2378,19 +2417,22 @@
         <v>2017</v>
       </c>
       <c r="B93">
-        <v>2.797254487856389</v>
+        <v>0.4354094579008074</v>
+      </c>
+      <c r="C93">
+        <v>0.9042764578833693</v>
       </c>
       <c r="D93" t="s">
         <v>13</v>
       </c>
       <c r="E93">
-        <v>1241</v>
+        <v>1406</v>
       </c>
       <c r="F93">
-        <v>480</v>
+        <v>2368</v>
       </c>
       <c r="G93">
-        <v>1180</v>
+        <v>11429</v>
       </c>
     </row>
     <row r="94" spans="1:7">
@@ -2398,22 +2440,22 @@
         <v>2018</v>
       </c>
       <c r="B94">
-        <v>0.9723032069970845</v>
+        <v>0.2195331519404267</v>
       </c>
       <c r="C94">
-        <v>1.766949152542373</v>
+        <v>0.9056785370548605</v>
       </c>
       <c r="D94" t="s">
         <v>13</v>
       </c>
       <c r="E94">
-        <v>1451</v>
+        <v>1578</v>
       </c>
       <c r="F94">
-        <v>467</v>
+        <v>2285</v>
       </c>
       <c r="G94">
-        <v>1101</v>
+        <v>11058</v>
       </c>
     </row>
     <row r="95" spans="1:7">
@@ -2424,19 +2466,19 @@
         <v>0</v>
       </c>
       <c r="C95">
-        <v>1.752043596730245</v>
+        <v>0.9177066377283415</v>
       </c>
       <c r="D95" t="s">
         <v>13</v>
       </c>
       <c r="E95">
-        <v>1309</v>
+        <v>1469</v>
       </c>
       <c r="F95">
-        <v>425</v>
+        <v>2330</v>
       </c>
       <c r="G95">
-        <v>1045</v>
+        <v>11009</v>
       </c>
     </row>
     <row r="96" spans="1:7">
@@ -2447,19 +2489,19 @@
         <v>0</v>
       </c>
       <c r="C96">
-        <v>1.873684210526316</v>
+        <v>0.9332364429103461</v>
       </c>
       <c r="D96" t="s">
         <v>13</v>
       </c>
       <c r="E96">
-        <v>1360</v>
+        <v>1512</v>
       </c>
       <c r="F96">
-        <v>387</v>
+        <v>2280</v>
       </c>
       <c r="G96">
-        <v>985</v>
+        <v>11042</v>
       </c>
     </row>
     <row r="97" spans="1:7">
@@ -2470,19 +2512,19 @@
         <v>0</v>
       </c>
       <c r="C97">
-        <v>1.861928934010152</v>
+        <v>0.9386886433617099</v>
       </c>
       <c r="D97" t="s">
         <v>13</v>
       </c>
       <c r="E97">
-        <v>1263</v>
+        <v>1335</v>
       </c>
       <c r="F97">
-        <v>431</v>
+        <v>2240</v>
       </c>
       <c r="G97">
-        <v>1002</v>
+        <v>11270</v>
       </c>
     </row>
     <row r="98" spans="1:7">
@@ -2493,19 +2535,19 @@
         <v>0</v>
       </c>
       <c r="C98">
-        <v>1.917165668662675</v>
+        <v>0.9204968944099379</v>
       </c>
       <c r="D98" t="s">
         <v>13</v>
       </c>
       <c r="E98">
-        <v>1315</v>
+        <v>1487</v>
       </c>
       <c r="F98">
-        <v>383</v>
+        <v>2143</v>
       </c>
       <c r="G98">
-        <v>989</v>
+        <v>11030</v>
       </c>
     </row>
     <row r="99" spans="1:7">
@@ -2516,121 +2558,154 @@
         <v>0</v>
       </c>
       <c r="C99">
-        <v>1.845298281092012</v>
+        <v>0.9485040797824116</v>
       </c>
       <c r="D99" t="s">
         <v>13</v>
       </c>
       <c r="E99">
-        <v>1334</v>
+        <v>1533</v>
       </c>
       <c r="F99">
-        <v>384</v>
+        <v>2084</v>
       </c>
       <c r="G99">
-        <v>875</v>
+        <v>11013</v>
       </c>
     </row>
     <row r="100" spans="1:7">
       <c r="A100">
         <v>2010</v>
       </c>
+      <c r="B100">
+        <v>1.214076246334311</v>
+      </c>
       <c r="D100" t="s">
         <v>14</v>
       </c>
       <c r="E100">
-        <v>354</v>
+        <v>31</v>
       </c>
       <c r="F100">
-        <v>0</v>
+        <v>170</v>
       </c>
       <c r="G100">
-        <v>0</v>
+        <v>865</v>
       </c>
     </row>
     <row r="101" spans="1:7">
       <c r="A101">
         <v>2011</v>
       </c>
+      <c r="B101">
+        <v>0.8426966292134831</v>
+      </c>
+      <c r="C101">
+        <v>1.064739884393064</v>
+      </c>
       <c r="D101" t="s">
         <v>14</v>
       </c>
       <c r="E101">
-        <v>346</v>
+        <v>121</v>
       </c>
       <c r="F101">
-        <v>0</v>
+        <v>171</v>
       </c>
       <c r="G101">
-        <v>0</v>
+        <v>971</v>
       </c>
     </row>
     <row r="102" spans="1:7">
       <c r="A102">
         <v>2012</v>
       </c>
+      <c r="B102">
+        <v>0.7888513513513513</v>
+      </c>
+      <c r="C102">
+        <v>0.9258496395468589</v>
+      </c>
       <c r="D102" t="s">
         <v>14</v>
       </c>
       <c r="E102">
-        <v>353</v>
+        <v>124</v>
       </c>
       <c r="F102">
-        <v>0</v>
+        <v>193</v>
       </c>
       <c r="G102">
-        <v>0</v>
+        <v>968</v>
       </c>
     </row>
     <row r="103" spans="1:7">
       <c r="A103">
         <v>2013</v>
       </c>
+      <c r="B103">
+        <v>0.7432216905901117</v>
+      </c>
+      <c r="C103">
+        <v>0.987603305785124</v>
+      </c>
       <c r="D103" t="s">
         <v>14</v>
       </c>
       <c r="E103">
-        <v>340</v>
+        <v>136</v>
       </c>
       <c r="F103">
-        <v>0</v>
+        <v>228</v>
       </c>
       <c r="G103">
-        <v>0</v>
+        <v>1048</v>
       </c>
     </row>
     <row r="104" spans="1:7">
       <c r="A104">
         <v>2014</v>
       </c>
+      <c r="B104">
+        <v>0.6642011834319527</v>
+      </c>
+      <c r="C104">
+        <v>0.9284351145038168</v>
+      </c>
       <c r="D104" t="s">
         <v>14</v>
       </c>
       <c r="E104">
-        <v>378</v>
+        <v>136</v>
       </c>
       <c r="F104">
-        <v>0</v>
+        <v>206</v>
       </c>
       <c r="G104">
-        <v>0</v>
+        <v>1043</v>
       </c>
     </row>
     <row r="105" spans="1:7">
       <c r="A105">
         <v>2015</v>
       </c>
+      <c r="B105">
+        <v>0.7443946188340808</v>
+      </c>
+      <c r="C105">
+        <v>0.9808245445829339</v>
+      </c>
       <c r="D105" t="s">
         <v>14</v>
       </c>
       <c r="E105">
-        <v>368</v>
+        <v>123</v>
       </c>
       <c r="F105">
-        <v>0</v>
+        <v>242</v>
       </c>
       <c r="G105">
-        <v>0</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="106" spans="1:7">
@@ -2638,19 +2713,22 @@
         <v>2016</v>
       </c>
       <c r="B106">
-        <v>9.236641221374045</v>
+        <v>0.818830242510699</v>
+      </c>
+      <c r="C106">
+        <v>1.019264448336252</v>
       </c>
       <c r="D106" t="s">
         <v>14</v>
       </c>
       <c r="E106">
-        <v>374</v>
+        <v>141</v>
       </c>
       <c r="F106">
-        <v>0</v>
+        <v>221</v>
       </c>
       <c r="G106">
-        <v>0</v>
+        <v>1244</v>
       </c>
     </row>
     <row r="107" spans="1:7">
@@ -2658,19 +2736,22 @@
         <v>2017</v>
       </c>
       <c r="B107">
-        <v>3.348</v>
+        <v>0.5454545454545454</v>
+      </c>
+      <c r="C107">
+        <v>0.9003215434083601</v>
       </c>
       <c r="D107" t="s">
         <v>14</v>
       </c>
       <c r="E107">
-        <v>394</v>
+        <v>150</v>
       </c>
       <c r="F107">
-        <v>131</v>
+        <v>238</v>
       </c>
       <c r="G107">
-        <v>376</v>
+        <v>1208</v>
       </c>
     </row>
     <row r="108" spans="1:7">
@@ -2678,22 +2759,22 @@
         <v>2018</v>
       </c>
       <c r="B108">
-        <v>1.239193083573487</v>
+        <v>0.2723970944309927</v>
       </c>
       <c r="C108">
-        <v>1.75531914893617</v>
+        <v>0.9478476821192053</v>
       </c>
       <c r="D108" t="s">
         <v>14</v>
       </c>
       <c r="E108">
-        <v>443</v>
+        <v>159</v>
       </c>
       <c r="F108">
-        <v>119</v>
+        <v>333</v>
       </c>
       <c r="G108">
-        <v>336</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="109" spans="1:7">
@@ -2704,19 +2785,19 @@
         <v>0</v>
       </c>
       <c r="C109">
-        <v>1.636904761904762</v>
+        <v>0.9044730856709629</v>
       </c>
       <c r="D109" t="s">
         <v>14</v>
       </c>
       <c r="E109">
-        <v>359</v>
+        <v>158</v>
       </c>
       <c r="F109">
-        <v>97</v>
+        <v>255</v>
       </c>
       <c r="G109">
-        <v>288</v>
+        <v>1290</v>
       </c>
     </row>
     <row r="110" spans="1:7">
@@ -2727,19 +2808,19 @@
         <v>0</v>
       </c>
       <c r="C110">
-        <v>1.958333333333333</v>
+        <v>0.9558139534883721</v>
       </c>
       <c r="D110" t="s">
         <v>14</v>
       </c>
       <c r="E110">
-        <v>407</v>
+        <v>149</v>
       </c>
       <c r="F110">
-        <v>117</v>
+        <v>302</v>
       </c>
       <c r="G110">
-        <v>274</v>
+        <v>1386</v>
       </c>
     </row>
     <row r="111" spans="1:7">
@@ -2750,19 +2831,19 @@
         <v>0</v>
       </c>
       <c r="C111">
-        <v>2.029197080291971</v>
+        <v>0.9487734487734488</v>
       </c>
       <c r="D111" t="s">
         <v>14</v>
       </c>
       <c r="E111">
-        <v>373</v>
+        <v>142</v>
       </c>
       <c r="F111">
-        <v>144</v>
+        <v>354</v>
       </c>
       <c r="G111">
-        <v>327</v>
+        <v>1527</v>
       </c>
     </row>
     <row r="112" spans="1:7">
@@ -2773,19 +2854,19 @@
         <v>0</v>
       </c>
       <c r="C112">
-        <v>1.819571865443425</v>
+        <v>0.9685658153241651</v>
       </c>
       <c r="D112" t="s">
         <v>14</v>
       </c>
       <c r="E112">
-        <v>407</v>
+        <v>207</v>
       </c>
       <c r="F112">
-        <v>141</v>
+        <v>355</v>
       </c>
       <c r="G112">
-        <v>329</v>
+        <v>1627</v>
       </c>
     </row>
     <row r="113" spans="1:7">
@@ -2796,19 +2877,19 @@
         <v>0</v>
       </c>
       <c r="C113">
-        <v>1.838905775075988</v>
+        <v>0.9551321450522434</v>
       </c>
       <c r="D113" t="s">
         <v>14</v>
       </c>
       <c r="E113">
-        <v>430</v>
+        <v>225</v>
       </c>
       <c r="F113">
-        <v>128</v>
+        <v>361</v>
       </c>
       <c r="G113">
-        <v>303</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="114" spans="1:7">
@@ -2816,19 +2897,19 @@
         <v>2010</v>
       </c>
       <c r="B114">
-        <v>0.9270678290452903</v>
+        <v>1.166666666666667</v>
       </c>
       <c r="D114" t="s">
         <v>15</v>
       </c>
       <c r="E114">
-        <v>514</v>
+        <v>18</v>
       </c>
       <c r="F114">
-        <v>2258</v>
+        <v>74</v>
       </c>
       <c r="G114">
-        <v>10960</v>
+        <v>287</v>
       </c>
     </row>
     <row r="115" spans="1:7">
@@ -2836,22 +2917,22 @@
         <v>2011</v>
       </c>
       <c r="B115">
-        <v>0.6391826236067448</v>
+        <v>0.8354430379746836</v>
       </c>
       <c r="C115">
-        <v>0.9498175182481752</v>
+        <v>1.114982578397212</v>
       </c>
       <c r="D115" t="s">
         <v>15</v>
       </c>
       <c r="E115">
-        <v>1358</v>
+        <v>49</v>
       </c>
       <c r="F115">
-        <v>2445</v>
+        <v>40</v>
       </c>
       <c r="G115">
-        <v>11497</v>
+        <v>311</v>
       </c>
     </row>
     <row r="116" spans="1:7">
@@ -2859,22 +2940,22 @@
         <v>2012</v>
       </c>
       <c r="B116">
-        <v>0.6308258960192662</v>
+        <v>0.8581081081081081</v>
       </c>
       <c r="C116">
-        <v>0.9038009915630164</v>
+        <v>0.8553054662379421</v>
       </c>
       <c r="D116" t="s">
         <v>15</v>
       </c>
       <c r="E116">
-        <v>1442</v>
+        <v>39</v>
       </c>
       <c r="F116">
-        <v>2295</v>
+        <v>44</v>
       </c>
       <c r="G116">
-        <v>11244</v>
+        <v>271</v>
       </c>
     </row>
     <row r="117" spans="1:7">
@@ -2882,22 +2963,22 @@
         <v>2013</v>
       </c>
       <c r="B117">
-        <v>0.665936313175577</v>
+        <v>0.7911392405063291</v>
       </c>
       <c r="C117">
-        <v>0.9447705442902882</v>
+        <v>0.959409594095941</v>
       </c>
       <c r="D117" t="s">
         <v>15</v>
       </c>
       <c r="E117">
-        <v>1501</v>
+        <v>53</v>
       </c>
       <c r="F117">
-        <v>2319</v>
+        <v>64</v>
       </c>
       <c r="G117">
-        <v>11441</v>
+        <v>271</v>
       </c>
     </row>
     <row r="118" spans="1:7">
@@ -2905,22 +2986,22 @@
         <v>2014</v>
       </c>
       <c r="B118">
-        <v>0.6342395297575312</v>
+        <v>0.7076023391812866</v>
       </c>
       <c r="C118">
-        <v>0.9562101214928765</v>
+        <v>0.955719557195572</v>
       </c>
       <c r="D118" t="s">
         <v>15</v>
       </c>
       <c r="E118">
-        <v>1462</v>
+        <v>41</v>
       </c>
       <c r="F118">
-        <v>2232</v>
+        <v>50</v>
       </c>
       <c r="G118">
-        <v>11710</v>
+        <v>268</v>
       </c>
     </row>
     <row r="119" spans="1:7">
@@ -2928,22 +3009,22 @@
         <v>2015</v>
       </c>
       <c r="B119">
-        <v>0.6402718274486631</v>
+        <v>0.676923076923077</v>
       </c>
       <c r="C119">
-        <v>0.9151152860802733</v>
+        <v>0.9328358208955224</v>
       </c>
       <c r="D119" t="s">
         <v>15</v>
       </c>
       <c r="E119">
-        <v>1465</v>
+        <v>41</v>
       </c>
       <c r="F119">
-        <v>2254</v>
+        <v>57</v>
       </c>
       <c r="G119">
-        <v>11505</v>
+        <v>266</v>
       </c>
     </row>
     <row r="120" spans="1:7">
@@ -2951,22 +3032,22 @@
         <v>2016</v>
       </c>
       <c r="B120">
-        <v>0.6307023895727734</v>
+        <v>0.5234375</v>
       </c>
       <c r="C120">
-        <v>0.937070838765754</v>
+        <v>0.8082706766917294</v>
       </c>
       <c r="D120" t="s">
         <v>15</v>
       </c>
       <c r="E120">
-        <v>1489</v>
+        <v>41</v>
       </c>
       <c r="F120">
-        <v>2283</v>
+        <v>88</v>
       </c>
       <c r="G120">
-        <v>11575</v>
+        <v>262</v>
       </c>
     </row>
     <row r="121" spans="1:7">
@@ -2974,22 +3055,22 @@
         <v>2017</v>
       </c>
       <c r="B121">
-        <v>0.4354094579008074</v>
+        <v>0.3121019108280255</v>
       </c>
       <c r="C121">
-        <v>0.9042764578833693</v>
+        <v>1.072519083969466</v>
       </c>
       <c r="D121" t="s">
         <v>15</v>
       </c>
       <c r="E121">
-        <v>1406</v>
+        <v>51</v>
       </c>
       <c r="F121">
-        <v>2368</v>
+        <v>111</v>
       </c>
       <c r="G121">
-        <v>11429</v>
+        <v>341</v>
       </c>
     </row>
     <row r="122" spans="1:7">
@@ -2997,22 +3078,22 @@
         <v>2018</v>
       </c>
       <c r="B122">
-        <v>0.2195331519404267</v>
+        <v>0.1522388059701492</v>
       </c>
       <c r="C122">
-        <v>0.9056785370548605</v>
+        <v>0.9442815249266863</v>
       </c>
       <c r="D122" t="s">
         <v>15</v>
       </c>
       <c r="E122">
-        <v>1578</v>
+        <v>40</v>
       </c>
       <c r="F122">
-        <v>2285</v>
+        <v>115</v>
       </c>
       <c r="G122">
-        <v>11058</v>
+        <v>397</v>
       </c>
     </row>
     <row r="123" spans="1:7">
@@ -3023,19 +3104,19 @@
         <v>0</v>
       </c>
       <c r="C123">
-        <v>0.9177066377283415</v>
+        <v>0.8261964735516373</v>
       </c>
       <c r="D123" t="s">
         <v>15</v>
       </c>
       <c r="E123">
-        <v>1469</v>
+        <v>36</v>
       </c>
       <c r="F123">
-        <v>2330</v>
+        <v>109</v>
       </c>
       <c r="G123">
-        <v>11009</v>
+        <v>401</v>
       </c>
     </row>
     <row r="124" spans="1:7">
@@ -3046,19 +3127,19 @@
         <v>0</v>
       </c>
       <c r="C124">
-        <v>0.9332364429103461</v>
+        <v>0.9226932668329177</v>
       </c>
       <c r="D124" t="s">
         <v>15</v>
       </c>
       <c r="E124">
-        <v>1512</v>
+        <v>49</v>
       </c>
       <c r="F124">
-        <v>2280</v>
+        <v>106</v>
       </c>
       <c r="G124">
-        <v>11042</v>
+        <v>427</v>
       </c>
     </row>
     <row r="125" spans="1:7">
@@ -3069,19 +3150,19 @@
         <v>0</v>
       </c>
       <c r="C125">
-        <v>0.9386886433617099</v>
+        <v>0.8618266978922716</v>
       </c>
       <c r="D125" t="s">
         <v>15</v>
       </c>
       <c r="E125">
-        <v>1335</v>
+        <v>36</v>
       </c>
       <c r="F125">
-        <v>2240</v>
+        <v>111</v>
       </c>
       <c r="G125">
-        <v>11270</v>
+        <v>443</v>
       </c>
     </row>
     <row r="126" spans="1:7">
@@ -3092,19 +3173,19 @@
         <v>0</v>
       </c>
       <c r="C126">
-        <v>0.9204968944099379</v>
+        <v>0.8848758465011287</v>
       </c>
       <c r="D126" t="s">
         <v>15</v>
       </c>
       <c r="E126">
-        <v>1487</v>
+        <v>47</v>
       </c>
       <c r="F126">
-        <v>2143</v>
+        <v>127</v>
       </c>
       <c r="G126">
-        <v>11030</v>
+        <v>472</v>
       </c>
     </row>
     <row r="127" spans="1:7">
@@ -3115,19 +3196,19 @@
         <v>0</v>
       </c>
       <c r="C127">
-        <v>0.9485040797824116</v>
+        <v>0.902542372881356</v>
       </c>
       <c r="D127" t="s">
         <v>15</v>
       </c>
       <c r="E127">
-        <v>1533</v>
+        <v>51</v>
       </c>
       <c r="F127">
-        <v>2084</v>
+        <v>109</v>
       </c>
       <c r="G127">
-        <v>11013</v>
+        <v>484</v>
       </c>
     </row>
     <row r="128" spans="1:7">
@@ -3135,19 +3216,19 @@
         <v>2010</v>
       </c>
       <c r="B128">
-        <v>1.214076246334311</v>
+        <v>1.252525252525253</v>
       </c>
       <c r="D128" t="s">
         <v>16</v>
       </c>
       <c r="E128">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F128">
-        <v>170</v>
+        <v>131</v>
       </c>
       <c r="G128">
-        <v>865</v>
+        <v>671</v>
       </c>
     </row>
     <row r="129" spans="1:7">
@@ -3155,22 +3236,22 @@
         <v>2011</v>
       </c>
       <c r="B129">
-        <v>0.8426966292134831</v>
+        <v>0.9029345372460497</v>
       </c>
       <c r="C129">
-        <v>1.064739884393064</v>
+        <v>0.9299552906110283</v>
       </c>
       <c r="D129" t="s">
         <v>16</v>
       </c>
       <c r="E129">
-        <v>121</v>
+        <v>77</v>
       </c>
       <c r="F129">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="G129">
-        <v>971</v>
+        <v>713</v>
       </c>
     </row>
     <row r="130" spans="1:7">
@@ -3178,22 +3259,22 @@
         <v>2012</v>
       </c>
       <c r="B130">
-        <v>0.7888513513513513</v>
+        <v>0.9683544303797469</v>
       </c>
       <c r="C130">
-        <v>0.9258496395468589</v>
+        <v>0.8849929873772791</v>
       </c>
       <c r="D130" t="s">
         <v>16</v>
       </c>
       <c r="E130">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="F130">
-        <v>193</v>
+        <v>146</v>
       </c>
       <c r="G130">
-        <v>968</v>
+        <v>668</v>
       </c>
     </row>
     <row r="131" spans="1:7">
@@ -3201,22 +3282,22 @@
         <v>2013</v>
       </c>
       <c r="B131">
-        <v>0.7432216905901117</v>
+        <v>0.9041353383458647</v>
       </c>
       <c r="C131">
-        <v>0.987603305785124</v>
+        <v>1.026946107784431</v>
       </c>
       <c r="D131" t="s">
         <v>16</v>
       </c>
       <c r="E131">
-        <v>136</v>
+        <v>97</v>
       </c>
       <c r="F131">
-        <v>228</v>
+        <v>162</v>
       </c>
       <c r="G131">
-        <v>1048</v>
+        <v>751</v>
       </c>
     </row>
     <row r="132" spans="1:7">
@@ -3224,22 +3305,22 @@
         <v>2014</v>
       </c>
       <c r="B132">
-        <v>0.6642011834319527</v>
+        <v>0.8174726989079563</v>
       </c>
       <c r="C132">
-        <v>0.9284351145038168</v>
+        <v>1.029294274300932</v>
       </c>
       <c r="D132" t="s">
         <v>16</v>
       </c>
       <c r="E132">
-        <v>136</v>
+        <v>109</v>
       </c>
       <c r="F132">
-        <v>206</v>
+        <v>224</v>
       </c>
       <c r="G132">
-        <v>1043</v>
+        <v>888</v>
       </c>
     </row>
     <row r="133" spans="1:7">
@@ -3247,22 +3328,22 @@
         <v>2015</v>
       </c>
       <c r="B133">
-        <v>0.7443946188340808</v>
+        <v>0.7434895833333334</v>
       </c>
       <c r="C133">
-        <v>0.9808245445829339</v>
+        <v>0.9403153153153153</v>
       </c>
       <c r="D133" t="s">
         <v>16</v>
       </c>
       <c r="E133">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F133">
-        <v>242</v>
+        <v>255</v>
       </c>
       <c r="G133">
-        <v>1142</v>
+        <v>968</v>
       </c>
     </row>
     <row r="134" spans="1:7">
@@ -3270,22 +3351,22 @@
         <v>2016</v>
       </c>
       <c r="B134">
-        <v>0.818830242510699</v>
+        <v>0.7244546498277842</v>
       </c>
       <c r="C134">
-        <v>1.019264448336252</v>
+        <v>0.9328512396694215</v>
       </c>
       <c r="D134" t="s">
         <v>16</v>
       </c>
       <c r="E134">
-        <v>141</v>
+        <v>115</v>
       </c>
       <c r="F134">
-        <v>221</v>
+        <v>289</v>
       </c>
       <c r="G134">
-        <v>1244</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="135" spans="1:7">
@@ -3293,22 +3374,22 @@
         <v>2017</v>
       </c>
       <c r="B135">
-        <v>0.5454545454545454</v>
+        <v>0.4591194968553459</v>
       </c>
       <c r="C135">
-        <v>0.9003215434083601</v>
+        <v>0.9795728876508821</v>
       </c>
       <c r="D135" t="s">
         <v>16</v>
       </c>
       <c r="E135">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="F135">
-        <v>238</v>
+        <v>327</v>
       </c>
       <c r="G135">
-        <v>1208</v>
+        <v>1247</v>
       </c>
     </row>
     <row r="136" spans="1:7">
@@ -3316,22 +3397,22 @@
         <v>2018</v>
       </c>
       <c r="B136">
-        <v>0.2723970944309927</v>
+        <v>0.2112950340798442</v>
       </c>
       <c r="C136">
-        <v>0.9478476821192053</v>
+        <v>0.917401764234162</v>
       </c>
       <c r="D136" t="s">
         <v>16</v>
       </c>
       <c r="E136">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="F136">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="G136">
-        <v>1319</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="137" spans="1:7">
@@ -3342,19 +3423,19 @@
         <v>0</v>
       </c>
       <c r="C137">
-        <v>0.9044730856709629</v>
+        <v>0.9459459459459459</v>
       </c>
       <c r="D137" t="s">
         <v>16</v>
       </c>
       <c r="E137">
-        <v>158</v>
+        <v>174</v>
       </c>
       <c r="F137">
-        <v>255</v>
+        <v>362</v>
       </c>
       <c r="G137">
-        <v>1290</v>
+        <v>1448</v>
       </c>
     </row>
     <row r="138" spans="1:7">
@@ -3365,19 +3446,19 @@
         <v>0</v>
       </c>
       <c r="C138">
-        <v>0.9558139534883721</v>
+        <v>0.9060773480662984</v>
       </c>
       <c r="D138" t="s">
         <v>16</v>
       </c>
       <c r="E138">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="F138">
-        <v>302</v>
+        <v>413</v>
       </c>
       <c r="G138">
-        <v>1386</v>
+        <v>1568</v>
       </c>
     </row>
     <row r="139" spans="1:7">
@@ -3388,19 +3469,19 @@
         <v>0</v>
       </c>
       <c r="C139">
-        <v>0.9487734487734488</v>
+        <v>0.9572704081632653</v>
       </c>
       <c r="D139" t="s">
         <v>16</v>
       </c>
       <c r="E139">
-        <v>142</v>
+        <v>193</v>
       </c>
       <c r="F139">
-        <v>354</v>
+        <v>460</v>
       </c>
       <c r="G139">
-        <v>1527</v>
+        <v>1768</v>
       </c>
     </row>
     <row r="140" spans="1:7">
@@ -3411,19 +3492,19 @@
         <v>0</v>
       </c>
       <c r="C140">
-        <v>0.9685658153241651</v>
+        <v>0.9010180995475113</v>
       </c>
       <c r="D140" t="s">
         <v>16</v>
       </c>
       <c r="E140">
-        <v>207</v>
+        <v>221</v>
       </c>
       <c r="F140">
         <v>355</v>
       </c>
       <c r="G140">
-        <v>1627</v>
+        <v>1727</v>
       </c>
     </row>
     <row r="141" spans="1:7">
@@ -3434,19 +3515,19 @@
         <v>0</v>
       </c>
       <c r="C141">
-        <v>0.9551321450522434</v>
+        <v>0.9270411117544876</v>
       </c>
       <c r="D141" t="s">
         <v>16</v>
       </c>
       <c r="E141">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="F141">
-        <v>361</v>
+        <v>418</v>
       </c>
       <c r="G141">
-        <v>1690</v>
+        <v>1802</v>
       </c>
     </row>
     <row r="142" spans="1:7">
@@ -3454,7 +3535,7 @@
         <v>2010</v>
       </c>
       <c r="B142">
-        <v>1.166666666666667</v>
+        <v>3.41025641025641</v>
       </c>
       <c r="D142" t="s">
         <v>17</v>
@@ -3463,10 +3544,10 @@
         <v>18</v>
       </c>
       <c r="F142">
-        <v>74</v>
+        <v>24</v>
       </c>
       <c r="G142">
-        <v>287</v>
+        <v>73</v>
       </c>
     </row>
     <row r="143" spans="1:7">
@@ -3474,10 +3555,10 @@
         <v>2011</v>
       </c>
       <c r="B143">
-        <v>0.8354430379746836</v>
+        <v>2.808510638297872</v>
       </c>
       <c r="C143">
-        <v>1.114982578397212</v>
+        <v>1.547945205479452</v>
       </c>
       <c r="D143" t="s">
         <v>17</v>
@@ -3486,10 +3567,10 @@
         <v>49</v>
       </c>
       <c r="F143">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="G143">
-        <v>311</v>
+        <v>79</v>
       </c>
     </row>
     <row r="144" spans="1:7">
@@ -3497,10 +3578,10 @@
         <v>2012</v>
       </c>
       <c r="B144">
-        <v>0.8581081081081081</v>
+        <v>3.96875</v>
       </c>
       <c r="C144">
-        <v>0.8553054662379421</v>
+        <v>1.265822784810127</v>
       </c>
       <c r="D144" t="s">
         <v>17</v>
@@ -3509,10 +3590,10 @@
         <v>39</v>
       </c>
       <c r="F144">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="G144">
-        <v>271</v>
+        <v>69</v>
       </c>
     </row>
     <row r="145" spans="1:7">
@@ -3520,10 +3601,10 @@
         <v>2013</v>
       </c>
       <c r="B145">
-        <v>0.7911392405063291</v>
+        <v>4.310344827586207</v>
       </c>
       <c r="C145">
-        <v>0.959409594095941</v>
+        <v>1.507246376811594</v>
       </c>
       <c r="D145" t="s">
         <v>17</v>
@@ -3532,10 +3613,10 @@
         <v>53</v>
       </c>
       <c r="F145">
-        <v>64</v>
+        <v>9</v>
       </c>
       <c r="G145">
-        <v>271</v>
+        <v>60</v>
       </c>
     </row>
     <row r="146" spans="1:7">
@@ -3543,10 +3624,10 @@
         <v>2014</v>
       </c>
       <c r="B146">
-        <v>0.7076023391812866</v>
+        <v>3.361111111111111</v>
       </c>
       <c r="C146">
-        <v>0.955719557195572</v>
+        <v>1.566666666666667</v>
       </c>
       <c r="D146" t="s">
         <v>17</v>
@@ -3555,10 +3636,10 @@
         <v>41</v>
       </c>
       <c r="F146">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="G146">
-        <v>268</v>
+        <v>65</v>
       </c>
     </row>
     <row r="147" spans="1:7">
@@ -3566,10 +3647,10 @@
         <v>2015</v>
       </c>
       <c r="B147">
-        <v>0.676923076923077</v>
+        <v>2.538461538461538</v>
       </c>
       <c r="C147">
-        <v>0.9328358208955224</v>
+        <v>1.307692307692308</v>
       </c>
       <c r="D147" t="s">
         <v>17</v>
@@ -3578,10 +3659,10 @@
         <v>41</v>
       </c>
       <c r="F147">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="G147">
-        <v>266</v>
+        <v>59</v>
       </c>
     </row>
     <row r="148" spans="1:7">
@@ -3589,10 +3670,10 @@
         <v>2016</v>
       </c>
       <c r="B148">
-        <v>0.5234375</v>
+        <v>2.03030303030303</v>
       </c>
       <c r="C148">
-        <v>0.8082706766917294</v>
+        <v>1.254237288135593</v>
       </c>
       <c r="D148" t="s">
         <v>17</v>
@@ -3601,10 +3682,10 @@
         <v>41</v>
       </c>
       <c r="F148">
-        <v>88</v>
+        <v>25</v>
       </c>
       <c r="G148">
-        <v>262</v>
+        <v>58</v>
       </c>
     </row>
     <row r="149" spans="1:7">
@@ -3612,10 +3693,10 @@
         <v>2017</v>
       </c>
       <c r="B149">
-        <v>0.3121019108280255</v>
+        <v>1.4</v>
       </c>
       <c r="C149">
-        <v>1.072519083969466</v>
+        <v>1.931034482758621</v>
       </c>
       <c r="D149" t="s">
         <v>17</v>
@@ -3624,10 +3705,10 @@
         <v>51</v>
       </c>
       <c r="F149">
-        <v>111</v>
+        <v>26</v>
       </c>
       <c r="G149">
-        <v>341</v>
+        <v>87</v>
       </c>
     </row>
     <row r="150" spans="1:7">
@@ -3635,10 +3716,10 @@
         <v>2018</v>
       </c>
       <c r="B150">
-        <v>0.1522388059701492</v>
+        <v>0.8360655737704918</v>
       </c>
       <c r="C150">
-        <v>0.9442815249266863</v>
+        <v>1.413793103448276</v>
       </c>
       <c r="D150" t="s">
         <v>17</v>
@@ -3647,10 +3728,10 @@
         <v>40</v>
       </c>
       <c r="F150">
-        <v>115</v>
+        <v>19</v>
       </c>
       <c r="G150">
-        <v>397</v>
+        <v>102</v>
       </c>
     </row>
     <row r="151" spans="1:7">
@@ -3661,7 +3742,7 @@
         <v>0</v>
       </c>
       <c r="C151">
-        <v>0.8261964735516373</v>
+        <v>1.107843137254902</v>
       </c>
       <c r="D151" t="s">
         <v>17</v>
@@ -3670,10 +3751,10 @@
         <v>36</v>
       </c>
       <c r="F151">
-        <v>109</v>
+        <v>16</v>
       </c>
       <c r="G151">
-        <v>401</v>
+        <v>93</v>
       </c>
     </row>
     <row r="152" spans="1:7">
@@ -3684,7 +3765,7 @@
         <v>0</v>
       </c>
       <c r="C152">
-        <v>0.9226932668329177</v>
+        <v>1.247311827956989</v>
       </c>
       <c r="D152" t="s">
         <v>17</v>
@@ -3693,10 +3774,10 @@
         <v>49</v>
       </c>
       <c r="F152">
+        <v>39</v>
+      </c>
+      <c r="G152">
         <v>106</v>
-      </c>
-      <c r="G152">
-        <v>427</v>
       </c>
     </row>
     <row r="153" spans="1:7">
@@ -3707,7 +3788,7 @@
         <v>0</v>
       </c>
       <c r="C153">
-        <v>0.8618266978922716</v>
+        <v>1.047169811320755</v>
       </c>
       <c r="D153" t="s">
         <v>17</v>
@@ -3716,10 +3797,10 @@
         <v>36</v>
       </c>
       <c r="F153">
+        <v>36</v>
+      </c>
+      <c r="G153">
         <v>111</v>
-      </c>
-      <c r="G153">
-        <v>443</v>
       </c>
     </row>
     <row r="154" spans="1:7">
@@ -3730,7 +3811,7 @@
         <v>0</v>
       </c>
       <c r="C154">
-        <v>0.8848758465011287</v>
+        <v>1.234234234234234</v>
       </c>
       <c r="D154" t="s">
         <v>17</v>
@@ -3739,10 +3820,10 @@
         <v>47</v>
       </c>
       <c r="F154">
-        <v>127</v>
+        <v>36</v>
       </c>
       <c r="G154">
-        <v>472</v>
+        <v>126</v>
       </c>
     </row>
     <row r="155" spans="1:7">
@@ -3753,7 +3834,7 @@
         <v>0</v>
       </c>
       <c r="C155">
-        <v>0.902542372881356</v>
+        <v>1.166666666666667</v>
       </c>
       <c r="D155" t="s">
         <v>17</v>
@@ -3762,10 +3843,10 @@
         <v>51</v>
       </c>
       <c r="F155">
-        <v>109</v>
+        <v>28</v>
       </c>
       <c r="G155">
-        <v>484</v>
+        <v>124</v>
       </c>
     </row>
     <row r="156" spans="1:7">
@@ -3773,19 +3854,19 @@
         <v>2010</v>
       </c>
       <c r="B156">
-        <v>1.252525252525253</v>
+        <v>6.369230769230769</v>
       </c>
       <c r="D156" t="s">
         <v>18</v>
       </c>
       <c r="E156">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F156">
-        <v>131</v>
+        <v>39</v>
       </c>
       <c r="G156">
-        <v>671</v>
+        <v>219</v>
       </c>
     </row>
     <row r="157" spans="1:7">
@@ -3793,22 +3874,22 @@
         <v>2011</v>
       </c>
       <c r="B157">
-        <v>0.9029345372460497</v>
+        <v>3.879310344827586</v>
       </c>
       <c r="C157">
-        <v>0.9299552906110283</v>
+        <v>1.45662100456621</v>
       </c>
       <c r="D157" t="s">
         <v>18</v>
       </c>
       <c r="E157">
-        <v>77</v>
+        <v>121</v>
       </c>
       <c r="F157">
-        <v>166</v>
+        <v>26</v>
       </c>
       <c r="G157">
-        <v>713</v>
+        <v>224</v>
       </c>
     </row>
     <row r="158" spans="1:7">
@@ -3816,22 +3897,22 @@
         <v>2012</v>
       </c>
       <c r="B158">
-        <v>0.9683544303797469</v>
+        <v>3.359712230215827</v>
       </c>
       <c r="C158">
-        <v>0.8849929873772791</v>
+        <v>1.348214285714286</v>
       </c>
       <c r="D158" t="s">
         <v>18</v>
       </c>
       <c r="E158">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="F158">
-        <v>146</v>
+        <v>51</v>
       </c>
       <c r="G158">
-        <v>668</v>
+        <v>229</v>
       </c>
     </row>
     <row r="159" spans="1:7">
@@ -3839,22 +3920,22 @@
         <v>2013</v>
       </c>
       <c r="B159">
-        <v>0.9041353383458647</v>
+        <v>3.106666666666666</v>
       </c>
       <c r="C159">
-        <v>1.026946107784431</v>
+        <v>1.436681222707423</v>
       </c>
       <c r="D159" t="s">
         <v>18</v>
       </c>
       <c r="E159">
-        <v>97</v>
+        <v>136</v>
       </c>
       <c r="F159">
-        <v>162</v>
+        <v>62</v>
       </c>
       <c r="G159">
-        <v>751</v>
+        <v>255</v>
       </c>
     </row>
     <row r="160" spans="1:7">
@@ -3862,22 +3943,22 @@
         <v>2014</v>
       </c>
       <c r="B160">
-        <v>0.8174726989079563</v>
+        <v>3.054421768707483</v>
       </c>
       <c r="C160">
-        <v>1.029294274300932</v>
+        <v>1.270588235294118</v>
       </c>
       <c r="D160" t="s">
         <v>18</v>
       </c>
       <c r="E160">
-        <v>109</v>
+        <v>136</v>
       </c>
       <c r="F160">
-        <v>224</v>
+        <v>37</v>
       </c>
       <c r="G160">
-        <v>888</v>
+        <v>225</v>
       </c>
     </row>
     <row r="161" spans="1:7">
@@ -3885,22 +3966,22 @@
         <v>2015</v>
       </c>
       <c r="B161">
-        <v>0.7434895833333334</v>
+        <v>3.171974522292994</v>
       </c>
       <c r="C161">
-        <v>0.9403153153153153</v>
+        <v>1.422222222222222</v>
       </c>
       <c r="D161" t="s">
         <v>18</v>
       </c>
       <c r="E161">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F161">
-        <v>255</v>
+        <v>48</v>
       </c>
       <c r="G161">
-        <v>968</v>
+        <v>245</v>
       </c>
     </row>
     <row r="162" spans="1:7">
@@ -3908,22 +3989,22 @@
         <v>2016</v>
       </c>
       <c r="B162">
-        <v>0.7244546498277842</v>
+        <v>3.242937853107345</v>
       </c>
       <c r="C162">
-        <v>0.9328512396694215</v>
+        <v>1.481632653061224</v>
       </c>
       <c r="D162" t="s">
         <v>18</v>
       </c>
       <c r="E162">
-        <v>115</v>
+        <v>141</v>
       </c>
       <c r="F162">
-        <v>289</v>
+        <v>72</v>
       </c>
       <c r="G162">
-        <v>1077</v>
+        <v>294</v>
       </c>
     </row>
     <row r="163" spans="1:7">
@@ -3931,22 +4012,22 @@
         <v>2017</v>
       </c>
       <c r="B163">
-        <v>0.4591194968553459</v>
+        <v>1.963636363636364</v>
       </c>
       <c r="C163">
-        <v>0.9795728876508821</v>
+        <v>1.30952380952381</v>
       </c>
       <c r="D163" t="s">
         <v>18</v>
       </c>
       <c r="E163">
-        <v>135</v>
+        <v>150</v>
       </c>
       <c r="F163">
-        <v>327</v>
+        <v>57</v>
       </c>
       <c r="G163">
-        <v>1247</v>
+        <v>292</v>
       </c>
     </row>
     <row r="164" spans="1:7">
@@ -3954,22 +4035,22 @@
         <v>2018</v>
       </c>
       <c r="B164">
-        <v>0.2112950340798442</v>
+        <v>1</v>
       </c>
       <c r="C164">
-        <v>0.917401764234162</v>
+        <v>1.397260273972603</v>
       </c>
       <c r="D164" t="s">
         <v>18</v>
       </c>
       <c r="E164">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="F164">
-        <v>338</v>
+        <v>91</v>
       </c>
       <c r="G164">
-        <v>1332</v>
+        <v>340</v>
       </c>
     </row>
     <row r="165" spans="1:7">
@@ -3980,19 +4061,19 @@
         <v>0</v>
       </c>
       <c r="C165">
-        <v>0.9459459459459459</v>
+        <v>1.214705882352941</v>
       </c>
       <c r="D165" t="s">
         <v>18</v>
       </c>
       <c r="E165">
-        <v>174</v>
+        <v>158</v>
       </c>
       <c r="F165">
-        <v>362</v>
+        <v>77</v>
       </c>
       <c r="G165">
-        <v>1448</v>
+        <v>332</v>
       </c>
     </row>
     <row r="166" spans="1:7">
@@ -4003,19 +4084,19 @@
         <v>0</v>
       </c>
       <c r="C166">
-        <v>0.9060773480662984</v>
+        <v>1.283132530120482</v>
       </c>
       <c r="D166" t="s">
         <v>18</v>
       </c>
       <c r="E166">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="F166">
-        <v>413</v>
+        <v>104</v>
       </c>
       <c r="G166">
-        <v>1568</v>
+        <v>381</v>
       </c>
     </row>
     <row r="167" spans="1:7">
@@ -4026,19 +4107,19 @@
         <v>0</v>
       </c>
       <c r="C167">
-        <v>0.9572704081632653</v>
+        <v>1.249343832020997</v>
       </c>
       <c r="D167" t="s">
         <v>18</v>
       </c>
       <c r="E167">
-        <v>193</v>
+        <v>142</v>
       </c>
       <c r="F167">
-        <v>460</v>
+        <v>117</v>
       </c>
       <c r="G167">
-        <v>1768</v>
+        <v>451</v>
       </c>
     </row>
     <row r="168" spans="1:7">
@@ -4049,19 +4130,19 @@
         <v>0</v>
       </c>
       <c r="C168">
-        <v>0.9010180995475113</v>
+        <v>1.321507760532151</v>
       </c>
       <c r="D168" t="s">
         <v>18</v>
       </c>
       <c r="E168">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="F168">
-        <v>355</v>
+        <v>113</v>
       </c>
       <c r="G168">
-        <v>1727</v>
+        <v>502</v>
       </c>
     </row>
     <row r="169" spans="1:7">
@@ -4072,19 +4153,338 @@
         <v>0</v>
       </c>
       <c r="C169">
-        <v>0.9270411117544876</v>
+        <v>1.258964143426295</v>
       </c>
       <c r="D169" t="s">
         <v>18</v>
       </c>
       <c r="E169">
+        <v>225</v>
+      </c>
+      <c r="F169">
+        <v>100</v>
+      </c>
+      <c r="G169">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7">
+      <c r="A170">
+        <v>2010</v>
+      </c>
+      <c r="B170">
+        <v>8.266666666666667</v>
+      </c>
+      <c r="D170" t="s">
+        <v>19</v>
+      </c>
+      <c r="E170">
+        <v>33</v>
+      </c>
+      <c r="F170">
+        <v>14</v>
+      </c>
+      <c r="G170">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="171" spans="1:7">
+      <c r="A171">
+        <v>2011</v>
+      </c>
+      <c r="B171">
+        <v>5.882352941176471</v>
+      </c>
+      <c r="C171">
+        <v>1.57843137254902</v>
+      </c>
+      <c r="D171" t="s">
+        <v>19</v>
+      </c>
+      <c r="E171">
+        <v>77</v>
+      </c>
+      <c r="F171">
+        <v>31</v>
+      </c>
+      <c r="G171">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="172" spans="1:7">
+      <c r="A172">
+        <v>2012</v>
+      </c>
+      <c r="B172">
+        <v>5.043956043956044</v>
+      </c>
+      <c r="C172">
+        <v>1.660869565217391</v>
+      </c>
+      <c r="D172" t="s">
+        <v>19</v>
+      </c>
+      <c r="E172">
+        <v>109</v>
+      </c>
+      <c r="F172">
+        <v>23</v>
+      </c>
+      <c r="G172">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="173" spans="1:7">
+      <c r="A173">
+        <v>2013</v>
+      </c>
+      <c r="B173">
+        <v>4.669902912621359</v>
+      </c>
+      <c r="C173">
+        <v>1.790476190476191</v>
+      </c>
+      <c r="D173" t="s">
+        <v>19</v>
+      </c>
+      <c r="E173">
+        <v>97</v>
+      </c>
+      <c r="F173">
+        <v>37</v>
+      </c>
+      <c r="G173">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7">
+      <c r="A174">
+        <v>2014</v>
+      </c>
+      <c r="B174">
+        <v>4.556521739130435</v>
+      </c>
+      <c r="C174">
+        <v>1.75</v>
+      </c>
+      <c r="D174" t="s">
+        <v>19</v>
+      </c>
+      <c r="E174">
+        <v>109</v>
+      </c>
+      <c r="F174">
+        <v>43</v>
+      </c>
+      <c r="G174">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="175" spans="1:7">
+      <c r="A175">
+        <v>2015</v>
+      </c>
+      <c r="B175">
+        <v>4.568</v>
+      </c>
+      <c r="C175">
+        <v>1.582278481012658</v>
+      </c>
+      <c r="D175" t="s">
+        <v>19</v>
+      </c>
+      <c r="E175">
+        <v>122</v>
+      </c>
+      <c r="F175">
+        <v>35</v>
+      </c>
+      <c r="G175">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="176" spans="1:7">
+      <c r="A176">
+        <v>2016</v>
+      </c>
+      <c r="B176">
+        <v>4.263513513513513</v>
+      </c>
+      <c r="C176">
+        <v>1.638036809815951</v>
+      </c>
+      <c r="D176" t="s">
+        <v>19</v>
+      </c>
+      <c r="E176">
+        <v>115</v>
+      </c>
+      <c r="F176">
+        <v>47</v>
+      </c>
+      <c r="G176">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="177" spans="1:7">
+      <c r="A177">
+        <v>2017</v>
+      </c>
+      <c r="B177">
+        <v>2.446927374301676</v>
+      </c>
+      <c r="C177">
+        <v>1.457286432160804</v>
+      </c>
+      <c r="D177" t="s">
+        <v>19</v>
+      </c>
+      <c r="E177">
+        <v>135</v>
+      </c>
+      <c r="F177">
+        <v>66</v>
+      </c>
+      <c r="G177">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7">
+      <c r="A178">
+        <v>2018</v>
+      </c>
+      <c r="B178">
+        <v>1.079601990049751</v>
+      </c>
+      <c r="C178">
+        <v>1.515837104072398</v>
+      </c>
+      <c r="D178" t="s">
+        <v>19</v>
+      </c>
+      <c r="E178">
+        <v>150</v>
+      </c>
+      <c r="F178">
+        <v>66</v>
+      </c>
+      <c r="G178">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="179" spans="1:7">
+      <c r="A179">
+        <v>2019</v>
+      </c>
+      <c r="B179">
+        <v>0</v>
+      </c>
+      <c r="C179">
+        <v>1.50996015936255</v>
+      </c>
+      <c r="D179" t="s">
+        <v>19</v>
+      </c>
+      <c r="E179">
+        <v>174</v>
+      </c>
+      <c r="F179">
+        <v>69</v>
+      </c>
+      <c r="G179">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="180" spans="1:7">
+      <c r="A180">
+        <v>2020</v>
+      </c>
+      <c r="B180">
+        <v>0</v>
+      </c>
+      <c r="C180">
+        <v>1.354014598540146</v>
+      </c>
+      <c r="D180" t="s">
+        <v>19</v>
+      </c>
+      <c r="E180">
+        <v>157</v>
+      </c>
+      <c r="F180">
+        <v>106</v>
+      </c>
+      <c r="G180">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="181" spans="1:7">
+      <c r="A181">
+        <v>2021</v>
+      </c>
+      <c r="B181">
+        <v>0</v>
+      </c>
+      <c r="C181">
+        <v>1.49375</v>
+      </c>
+      <c r="D181" t="s">
+        <v>19</v>
+      </c>
+      <c r="E181">
+        <v>193</v>
+      </c>
+      <c r="F181">
+        <v>153</v>
+      </c>
+      <c r="G181">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="182" spans="1:7">
+      <c r="A182">
+        <v>2022</v>
+      </c>
+      <c r="B182">
+        <v>0</v>
+      </c>
+      <c r="C182">
+        <v>1.248858447488584</v>
+      </c>
+      <c r="D182" t="s">
+        <v>19</v>
+      </c>
+      <c r="E182">
+        <v>221</v>
+      </c>
+      <c r="F182">
+        <v>91</v>
+      </c>
+      <c r="G182">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="183" spans="1:7">
+      <c r="A183">
+        <v>2023</v>
+      </c>
+      <c r="B183">
+        <v>0</v>
+      </c>
+      <c r="C183">
+        <v>1.290167865707434</v>
+      </c>
+      <c r="D183" t="s">
+        <v>19</v>
+      </c>
+      <c r="E183">
         <v>217</v>
       </c>
-      <c r="F169">
-        <v>418</v>
-      </c>
-      <c r="G169">
-        <v>1802</v>
+      <c r="F183">
+        <v>111</v>
+      </c>
+      <c r="G183">
+        <v>432</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed Issuw with incorect variable being used for degrees awarded for sex and race variables
</commit_message>
<xml_diff>
--- a/graphs/PCR_Retention_National.xlsx
+++ b/graphs/PCR_Retention_National.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="24">
   <si>
     <t>year</t>
   </si>
@@ -65,6 +65,18 @@
   </si>
   <si>
     <t>Hispanic</t>
+  </si>
+  <si>
+    <t>Native Hawaiian /Pacific islander</t>
+  </si>
+  <si>
+    <t>2 or more</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>Foreign</t>
   </si>
   <si>
     <t>Black Women</t>
@@ -431,7 +443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G183"/>
+  <dimension ref="A1:G239"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -3535,19 +3547,19 @@
         <v>2010</v>
       </c>
       <c r="B142">
-        <v>3.41025641025641</v>
+        <v>0.5</v>
       </c>
       <c r="D142" t="s">
         <v>17</v>
       </c>
       <c r="E142">
+        <v>0</v>
+      </c>
+      <c r="F142">
+        <v>3</v>
+      </c>
+      <c r="G142">
         <v>18</v>
-      </c>
-      <c r="F142">
-        <v>24</v>
-      </c>
-      <c r="G142">
-        <v>73</v>
       </c>
     </row>
     <row r="143" spans="1:7">
@@ -3555,22 +3567,22 @@
         <v>2011</v>
       </c>
       <c r="B143">
-        <v>2.808510638297872</v>
+        <v>0.4117647058823529</v>
       </c>
       <c r="C143">
-        <v>1.547945205479452</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="D143" t="s">
         <v>17</v>
       </c>
       <c r="E143">
-        <v>49</v>
+        <v>1</v>
       </c>
       <c r="F143">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G143">
-        <v>79</v>
+        <v>26</v>
       </c>
     </row>
     <row r="144" spans="1:7">
@@ -3578,22 +3590,22 @@
         <v>2012</v>
       </c>
       <c r="B144">
-        <v>3.96875</v>
+        <v>0.4375</v>
       </c>
       <c r="C144">
-        <v>1.265822784810127</v>
+        <v>0.6538461538461539</v>
       </c>
       <c r="D144" t="s">
         <v>17</v>
       </c>
       <c r="E144">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="F144">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G144">
-        <v>69</v>
+        <v>19</v>
       </c>
     </row>
     <row r="145" spans="1:7">
@@ -3601,22 +3613,22 @@
         <v>2013</v>
       </c>
       <c r="B145">
-        <v>4.310344827586207</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="C145">
-        <v>1.507246376811594</v>
+        <v>0.8947368421052632</v>
       </c>
       <c r="D145" t="s">
         <v>17</v>
       </c>
       <c r="E145">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="F145">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G145">
-        <v>60</v>
+        <v>18</v>
       </c>
     </row>
     <row r="146" spans="1:7">
@@ -3624,22 +3636,22 @@
         <v>2014</v>
       </c>
       <c r="B146">
-        <v>3.361111111111111</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="C146">
-        <v>1.566666666666667</v>
+        <v>1.166666666666667</v>
       </c>
       <c r="D146" t="s">
         <v>17</v>
       </c>
       <c r="E146">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="F146">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G146">
-        <v>65</v>
+        <v>22</v>
       </c>
     </row>
     <row r="147" spans="1:7">
@@ -3647,22 +3659,22 @@
         <v>2015</v>
       </c>
       <c r="B147">
-        <v>2.538461538461538</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="C147">
-        <v>1.307692307692308</v>
+        <v>0.9545454545454546</v>
       </c>
       <c r="D147" t="s">
         <v>17</v>
       </c>
       <c r="E147">
-        <v>41</v>
+        <v>3</v>
       </c>
       <c r="F147">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="G147">
-        <v>59</v>
+        <v>26</v>
       </c>
     </row>
     <row r="148" spans="1:7">
@@ -3670,22 +3682,22 @@
         <v>2016</v>
       </c>
       <c r="B148">
-        <v>2.03030303030303</v>
+        <v>0.5</v>
       </c>
       <c r="C148">
-        <v>1.254237288135593</v>
+        <v>0.5384615384615384</v>
       </c>
       <c r="D148" t="s">
         <v>17</v>
       </c>
       <c r="E148">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="F148">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="G148">
-        <v>58</v>
+        <v>14</v>
       </c>
     </row>
     <row r="149" spans="1:7">
@@ -3693,22 +3705,22 @@
         <v>2017</v>
       </c>
       <c r="B149">
-        <v>1.4</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="C149">
-        <v>1.931034482758621</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="D149" t="s">
         <v>17</v>
       </c>
       <c r="E149">
-        <v>51</v>
+        <v>2</v>
       </c>
       <c r="F149">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="G149">
-        <v>87</v>
+        <v>8</v>
       </c>
     </row>
     <row r="150" spans="1:7">
@@ -3716,22 +3728,22 @@
         <v>2018</v>
       </c>
       <c r="B150">
-        <v>0.8360655737704918</v>
+        <v>0</v>
       </c>
       <c r="C150">
-        <v>1.413793103448276</v>
+        <v>0.875</v>
       </c>
       <c r="D150" t="s">
         <v>17</v>
       </c>
       <c r="E150">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="F150">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="G150">
-        <v>102</v>
+        <v>9</v>
       </c>
     </row>
     <row r="151" spans="1:7">
@@ -3742,19 +3754,19 @@
         <v>0</v>
       </c>
       <c r="C151">
-        <v>1.107843137254902</v>
+        <v>0.7777777777777778</v>
       </c>
       <c r="D151" t="s">
         <v>17</v>
       </c>
       <c r="E151">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="F151">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="G151">
-        <v>93</v>
+        <v>8</v>
       </c>
     </row>
     <row r="152" spans="1:7">
@@ -3765,19 +3777,19 @@
         <v>0</v>
       </c>
       <c r="C152">
-        <v>1.247311827956989</v>
+        <v>0.625</v>
       </c>
       <c r="D152" t="s">
         <v>17</v>
       </c>
       <c r="E152">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="F152">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="G152">
-        <v>106</v>
+        <v>5</v>
       </c>
     </row>
     <row r="153" spans="1:7">
@@ -3788,19 +3800,19 @@
         <v>0</v>
       </c>
       <c r="C153">
-        <v>1.047169811320755</v>
+        <v>0.6</v>
       </c>
       <c r="D153" t="s">
         <v>17</v>
       </c>
       <c r="E153">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="F153">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="G153">
-        <v>111</v>
+        <v>0</v>
       </c>
     </row>
     <row r="154" spans="1:7">
@@ -3810,20 +3822,17 @@
       <c r="B154">
         <v>0</v>
       </c>
-      <c r="C154">
-        <v>1.234234234234234</v>
-      </c>
       <c r="D154" t="s">
         <v>17</v>
       </c>
       <c r="E154">
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="F154">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="G154">
-        <v>126</v>
+        <v>3</v>
       </c>
     </row>
     <row r="155" spans="1:7">
@@ -3834,19 +3843,19 @@
         <v>0</v>
       </c>
       <c r="C155">
-        <v>1.166666666666667</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="D155" t="s">
         <v>17</v>
       </c>
       <c r="E155">
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="F155">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="G155">
-        <v>124</v>
+        <v>1</v>
       </c>
     </row>
     <row r="156" spans="1:7">
@@ -3854,19 +3863,19 @@
         <v>2010</v>
       </c>
       <c r="B156">
-        <v>6.369230769230769</v>
+        <v>1.11304347826087</v>
       </c>
       <c r="D156" t="s">
         <v>18</v>
       </c>
       <c r="E156">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="F156">
-        <v>39</v>
+        <v>58</v>
       </c>
       <c r="G156">
-        <v>219</v>
+        <v>0</v>
       </c>
     </row>
     <row r="157" spans="1:7">
@@ -3874,22 +3883,19 @@
         <v>2011</v>
       </c>
       <c r="B157">
-        <v>3.879310344827586</v>
-      </c>
-      <c r="C157">
-        <v>1.45662100456621</v>
+        <v>0.9879518072289156</v>
       </c>
       <c r="D157" t="s">
         <v>18</v>
       </c>
       <c r="E157">
-        <v>121</v>
+        <v>15</v>
       </c>
       <c r="F157">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="G157">
-        <v>224</v>
+        <v>0</v>
       </c>
     </row>
     <row r="158" spans="1:7">
@@ -3897,22 +3903,19 @@
         <v>2012</v>
       </c>
       <c r="B158">
-        <v>3.359712230215827</v>
-      </c>
-      <c r="C158">
-        <v>1.348214285714286</v>
+        <v>0.8944723618090452</v>
       </c>
       <c r="D158" t="s">
         <v>18</v>
       </c>
       <c r="E158">
-        <v>124</v>
+        <v>27</v>
       </c>
       <c r="F158">
         <v>51</v>
       </c>
       <c r="G158">
-        <v>229</v>
+        <v>0</v>
       </c>
     </row>
     <row r="159" spans="1:7">
@@ -3920,22 +3923,19 @@
         <v>2013</v>
       </c>
       <c r="B159">
-        <v>3.106666666666666</v>
-      </c>
-      <c r="C159">
-        <v>1.436681222707423</v>
+        <v>0.9178082191780822</v>
       </c>
       <c r="D159" t="s">
         <v>18</v>
       </c>
       <c r="E159">
-        <v>136</v>
+        <v>48</v>
       </c>
       <c r="F159">
-        <v>62</v>
+        <v>91</v>
       </c>
       <c r="G159">
-        <v>255</v>
+        <v>0</v>
       </c>
     </row>
     <row r="160" spans="1:7">
@@ -3943,22 +3943,19 @@
         <v>2014</v>
       </c>
       <c r="B160">
-        <v>3.054421768707483</v>
-      </c>
-      <c r="C160">
-        <v>1.270588235294118</v>
+        <v>0.7490494296577946</v>
       </c>
       <c r="D160" t="s">
         <v>18</v>
       </c>
       <c r="E160">
-        <v>136</v>
+        <v>34</v>
       </c>
       <c r="F160">
-        <v>37</v>
+        <v>77</v>
       </c>
       <c r="G160">
-        <v>225</v>
+        <v>0</v>
       </c>
     </row>
     <row r="161" spans="1:7">
@@ -3966,22 +3963,19 @@
         <v>2015</v>
       </c>
       <c r="B161">
-        <v>3.171974522292994</v>
-      </c>
-      <c r="C161">
-        <v>1.422222222222222</v>
+        <v>0.8223938223938224</v>
       </c>
       <c r="D161" t="s">
         <v>18</v>
       </c>
       <c r="E161">
-        <v>123</v>
+        <v>33</v>
       </c>
       <c r="F161">
-        <v>48</v>
+        <v>95</v>
       </c>
       <c r="G161">
-        <v>245</v>
+        <v>0</v>
       </c>
     </row>
     <row r="162" spans="1:7">
@@ -3989,22 +3983,19 @@
         <v>2016</v>
       </c>
       <c r="B162">
-        <v>3.242937853107345</v>
-      </c>
-      <c r="C162">
-        <v>1.481632653061224</v>
+        <v>0.7174603174603175</v>
       </c>
       <c r="D162" t="s">
         <v>18</v>
       </c>
       <c r="E162">
-        <v>141</v>
+        <v>47</v>
       </c>
       <c r="F162">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="G162">
-        <v>294</v>
+        <v>0</v>
       </c>
     </row>
     <row r="163" spans="1:7">
@@ -4012,22 +4003,19 @@
         <v>2017</v>
       </c>
       <c r="B163">
-        <v>1.963636363636364</v>
-      </c>
-      <c r="C163">
-        <v>1.30952380952381</v>
+        <v>0.4573863636363636</v>
       </c>
       <c r="D163" t="s">
         <v>18</v>
       </c>
       <c r="E163">
-        <v>150</v>
+        <v>48</v>
       </c>
       <c r="F163">
-        <v>57</v>
+        <v>133</v>
       </c>
       <c r="G163">
-        <v>292</v>
+        <v>510</v>
       </c>
     </row>
     <row r="164" spans="1:7">
@@ -4035,22 +4023,22 @@
         <v>2018</v>
       </c>
       <c r="B164">
-        <v>1</v>
+        <v>0.208955223880597</v>
       </c>
       <c r="C164">
-        <v>1.397260273972603</v>
+        <v>0.8980392156862745</v>
       </c>
       <c r="D164" t="s">
         <v>18</v>
       </c>
       <c r="E164">
-        <v>159</v>
+        <v>69</v>
       </c>
       <c r="F164">
-        <v>91</v>
+        <v>132</v>
       </c>
       <c r="G164">
-        <v>340</v>
+        <v>521</v>
       </c>
     </row>
     <row r="165" spans="1:7">
@@ -4061,19 +4049,19 @@
         <v>0</v>
       </c>
       <c r="C165">
-        <v>1.214705882352941</v>
+        <v>0.8637236084452975</v>
       </c>
       <c r="D165" t="s">
         <v>18</v>
       </c>
       <c r="E165">
-        <v>158</v>
+        <v>61</v>
       </c>
       <c r="F165">
-        <v>77</v>
+        <v>137</v>
       </c>
       <c r="G165">
-        <v>332</v>
+        <v>526</v>
       </c>
     </row>
     <row r="166" spans="1:7">
@@ -4084,19 +4072,19 @@
         <v>0</v>
       </c>
       <c r="C166">
-        <v>1.283132530120482</v>
+        <v>0.9847908745247148</v>
       </c>
       <c r="D166" t="s">
         <v>18</v>
       </c>
       <c r="E166">
-        <v>149</v>
+        <v>71</v>
       </c>
       <c r="F166">
-        <v>104</v>
+        <v>143</v>
       </c>
       <c r="G166">
-        <v>381</v>
+        <v>590</v>
       </c>
     </row>
     <row r="167" spans="1:7">
@@ -4107,19 +4095,19 @@
         <v>0</v>
       </c>
       <c r="C167">
-        <v>1.249343832020997</v>
+        <v>0.9355932203389831</v>
       </c>
       <c r="D167" t="s">
         <v>18</v>
       </c>
       <c r="E167">
-        <v>142</v>
+        <v>65</v>
       </c>
       <c r="F167">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="G167">
-        <v>451</v>
+        <v>608</v>
       </c>
     </row>
     <row r="168" spans="1:7">
@@ -4130,19 +4118,19 @@
         <v>0</v>
       </c>
       <c r="C168">
-        <v>1.321507760532151</v>
+        <v>0.9473684210526315</v>
       </c>
       <c r="D168" t="s">
         <v>18</v>
       </c>
       <c r="E168">
-        <v>207</v>
+        <v>77</v>
       </c>
       <c r="F168">
-        <v>113</v>
+        <v>151</v>
       </c>
       <c r="G168">
-        <v>502</v>
+        <v>650</v>
       </c>
     </row>
     <row r="169" spans="1:7">
@@ -4153,19 +4141,19 @@
         <v>0</v>
       </c>
       <c r="C169">
-        <v>1.258964143426295</v>
+        <v>1.026153846153846</v>
       </c>
       <c r="D169" t="s">
         <v>18</v>
       </c>
       <c r="E169">
-        <v>225</v>
+        <v>84</v>
       </c>
       <c r="F169">
-        <v>100</v>
+        <v>174</v>
       </c>
       <c r="G169">
-        <v>507</v>
+        <v>757</v>
       </c>
     </row>
     <row r="170" spans="1:7">
@@ -4173,19 +4161,19 @@
         <v>2010</v>
       </c>
       <c r="B170">
-        <v>8.266666666666667</v>
+        <v>1.198924731182796</v>
       </c>
       <c r="D170" t="s">
         <v>19</v>
       </c>
       <c r="E170">
-        <v>33</v>
+        <v>215</v>
       </c>
       <c r="F170">
-        <v>14</v>
+        <v>205</v>
       </c>
       <c r="G170">
-        <v>102</v>
+        <v>0</v>
       </c>
     </row>
     <row r="171" spans="1:7">
@@ -4193,22 +4181,19 @@
         <v>2011</v>
       </c>
       <c r="B171">
-        <v>5.882352941176471</v>
-      </c>
-      <c r="C171">
-        <v>1.57843137254902</v>
+        <v>0.6881720430107527</v>
       </c>
       <c r="D171" t="s">
         <v>19</v>
       </c>
       <c r="E171">
-        <v>77</v>
+        <v>191</v>
       </c>
       <c r="F171">
-        <v>31</v>
+        <v>167</v>
       </c>
       <c r="G171">
-        <v>115</v>
+        <v>0</v>
       </c>
     </row>
     <row r="172" spans="1:7">
@@ -4216,22 +4201,19 @@
         <v>2012</v>
       </c>
       <c r="B172">
-        <v>5.043956043956044</v>
-      </c>
-      <c r="C172">
-        <v>1.660869565217391</v>
+        <v>0.7320388349514563</v>
       </c>
       <c r="D172" t="s">
         <v>19</v>
       </c>
       <c r="E172">
-        <v>109</v>
+        <v>178</v>
       </c>
       <c r="F172">
-        <v>23</v>
+        <v>186</v>
       </c>
       <c r="G172">
-        <v>105</v>
+        <v>0</v>
       </c>
     </row>
     <row r="173" spans="1:7">
@@ -4239,22 +4221,19 @@
         <v>2013</v>
       </c>
       <c r="B173">
-        <v>4.669902912621359</v>
-      </c>
-      <c r="C173">
-        <v>1.790476190476191</v>
+        <v>0.7956989247311828</v>
       </c>
       <c r="D173" t="s">
         <v>19</v>
       </c>
       <c r="E173">
-        <v>97</v>
+        <v>179</v>
       </c>
       <c r="F173">
-        <v>37</v>
+        <v>162</v>
       </c>
       <c r="G173">
-        <v>128</v>
+        <v>0</v>
       </c>
     </row>
     <row r="174" spans="1:7">
@@ -4262,22 +4241,19 @@
         <v>2014</v>
       </c>
       <c r="B174">
-        <v>4.556521739130435</v>
-      </c>
-      <c r="C174">
-        <v>1.75</v>
+        <v>0.7832167832167832</v>
       </c>
       <c r="D174" t="s">
         <v>19</v>
       </c>
       <c r="E174">
-        <v>109</v>
+        <v>157</v>
       </c>
       <c r="F174">
-        <v>43</v>
+        <v>117</v>
       </c>
       <c r="G174">
-        <v>158</v>
+        <v>0</v>
       </c>
     </row>
     <row r="175" spans="1:7">
@@ -4285,22 +4261,19 @@
         <v>2015</v>
       </c>
       <c r="B175">
-        <v>4.568</v>
-      </c>
-      <c r="C175">
-        <v>1.582278481012658</v>
+        <v>0.776595744680851</v>
       </c>
       <c r="D175" t="s">
         <v>19</v>
       </c>
       <c r="E175">
-        <v>122</v>
+        <v>181</v>
       </c>
       <c r="F175">
-        <v>35</v>
+        <v>150</v>
       </c>
       <c r="G175">
-        <v>163</v>
+        <v>0</v>
       </c>
     </row>
     <row r="176" spans="1:7">
@@ -4308,22 +4281,19 @@
         <v>2016</v>
       </c>
       <c r="B176">
-        <v>4.263513513513513</v>
-      </c>
-      <c r="C176">
-        <v>1.638036809815951</v>
+        <v>0.6953316953316954</v>
       </c>
       <c r="D176" t="s">
         <v>19</v>
       </c>
       <c r="E176">
-        <v>115</v>
+        <v>147</v>
       </c>
       <c r="F176">
-        <v>47</v>
+        <v>109</v>
       </c>
       <c r="G176">
-        <v>199</v>
+        <v>0</v>
       </c>
     </row>
     <row r="177" spans="1:7">
@@ -4331,22 +4301,19 @@
         <v>2017</v>
       </c>
       <c r="B177">
-        <v>2.446927374301676</v>
-      </c>
-      <c r="C177">
-        <v>1.457286432160804</v>
+        <v>0.5063938618925832</v>
       </c>
       <c r="D177" t="s">
         <v>19</v>
       </c>
       <c r="E177">
-        <v>135</v>
+        <v>118</v>
       </c>
       <c r="F177">
-        <v>66</v>
+        <v>148</v>
       </c>
       <c r="G177">
-        <v>221</v>
+        <v>773</v>
       </c>
     </row>
     <row r="178" spans="1:7">
@@ -4354,22 +4321,22 @@
         <v>2018</v>
       </c>
       <c r="B178">
-        <v>1.079601990049751</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="C178">
-        <v>1.515837104072398</v>
+        <v>0.8758085381630013</v>
       </c>
       <c r="D178" t="s">
         <v>19</v>
       </c>
       <c r="E178">
-        <v>150</v>
+        <v>119</v>
       </c>
       <c r="F178">
-        <v>66</v>
+        <v>134</v>
       </c>
       <c r="G178">
-        <v>251</v>
+        <v>692</v>
       </c>
     </row>
     <row r="179" spans="1:7">
@@ -4380,19 +4347,19 @@
         <v>0</v>
       </c>
       <c r="C179">
-        <v>1.50996015936255</v>
+        <v>1.030346820809249</v>
       </c>
       <c r="D179" t="s">
         <v>19</v>
       </c>
       <c r="E179">
-        <v>174</v>
+        <v>140</v>
       </c>
       <c r="F179">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="G179">
-        <v>274</v>
+        <v>648</v>
       </c>
     </row>
     <row r="180" spans="1:7">
@@ -4403,19 +4370,19 @@
         <v>0</v>
       </c>
       <c r="C180">
-        <v>1.354014598540146</v>
+        <v>0.9583333333333334</v>
       </c>
       <c r="D180" t="s">
         <v>19</v>
       </c>
       <c r="E180">
-        <v>157</v>
+        <v>111</v>
       </c>
       <c r="F180">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="G180">
-        <v>320</v>
+        <v>630</v>
       </c>
     </row>
     <row r="181" spans="1:7">
@@ -4426,19 +4393,19 @@
         <v>0</v>
       </c>
       <c r="C181">
-        <v>1.49375</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="D181" t="s">
         <v>19</v>
       </c>
       <c r="E181">
-        <v>193</v>
+        <v>85</v>
       </c>
       <c r="F181">
-        <v>153</v>
+        <v>164</v>
       </c>
       <c r="G181">
-        <v>438</v>
+        <v>639</v>
       </c>
     </row>
     <row r="182" spans="1:7">
@@ -4449,19 +4416,19 @@
         <v>0</v>
       </c>
       <c r="C182">
-        <v>1.248858447488584</v>
+        <v>0.9342723004694836</v>
       </c>
       <c r="D182" t="s">
         <v>19</v>
       </c>
       <c r="E182">
-        <v>221</v>
+        <v>96</v>
       </c>
       <c r="F182">
-        <v>91</v>
+        <v>136</v>
       </c>
       <c r="G182">
-        <v>417</v>
+        <v>637</v>
       </c>
     </row>
     <row r="183" spans="1:7">
@@ -4472,18 +4439,1294 @@
         <v>0</v>
       </c>
       <c r="C183">
-        <v>1.290167865707434</v>
+        <v>1.003139717425432</v>
       </c>
       <c r="D183" t="s">
         <v>19</v>
       </c>
       <c r="E183">
+        <v>102</v>
+      </c>
+      <c r="F183">
+        <v>87</v>
+      </c>
+      <c r="G183">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="184" spans="1:7">
+      <c r="A184">
+        <v>2010</v>
+      </c>
+      <c r="B184">
+        <v>0.9302748126277538</v>
+      </c>
+      <c r="D184" t="s">
+        <v>20</v>
+      </c>
+      <c r="E184">
+        <v>1230</v>
+      </c>
+      <c r="F184">
+        <v>2119</v>
+      </c>
+      <c r="G184">
+        <v>11040</v>
+      </c>
+    </row>
+    <row r="185" spans="1:7">
+      <c r="A185">
+        <v>2011</v>
+      </c>
+      <c r="B185">
+        <v>0.6321993434795583</v>
+      </c>
+      <c r="C185">
+        <v>0.9295289855072464</v>
+      </c>
+      <c r="D185" t="s">
+        <v>20</v>
+      </c>
+      <c r="E185">
+        <v>1195</v>
+      </c>
+      <c r="F185">
+        <v>2284</v>
+      </c>
+      <c r="G185">
+        <v>11351</v>
+      </c>
+    </row>
+    <row r="186" spans="1:7">
+      <c r="A186">
+        <v>2012</v>
+      </c>
+      <c r="B186">
+        <v>0.6324621324621325</v>
+      </c>
+      <c r="C186">
+        <v>0.920271341732006</v>
+      </c>
+      <c r="D186" t="s">
+        <v>20</v>
+      </c>
+      <c r="E186">
+        <v>1330</v>
+      </c>
+      <c r="F186">
+        <v>2299</v>
+      </c>
+      <c r="G186">
+        <v>11415</v>
+      </c>
+    </row>
+    <row r="187" spans="1:7">
+      <c r="A187">
+        <v>2013</v>
+      </c>
+      <c r="B187">
+        <v>0.6249072287368265</v>
+      </c>
+      <c r="C187">
+        <v>0.9472623740692072</v>
+      </c>
+      <c r="D187" t="s">
+        <v>20</v>
+      </c>
+      <c r="E187">
+        <v>1277</v>
+      </c>
+      <c r="F187">
+        <v>2151</v>
+      </c>
+      <c r="G187">
+        <v>11687</v>
+      </c>
+    </row>
+    <row r="188" spans="1:7">
+      <c r="A188">
+        <v>2014</v>
+      </c>
+      <c r="B188">
+        <v>0.5917279146851131</v>
+      </c>
+      <c r="C188">
+        <v>0.9401043894925987</v>
+      </c>
+      <c r="D188" t="s">
+        <v>20</v>
+      </c>
+      <c r="E188">
+        <v>1308</v>
+      </c>
+      <c r="F188">
+        <v>2287</v>
+      </c>
+      <c r="G188">
+        <v>11966</v>
+      </c>
+    </row>
+    <row r="189" spans="1:7">
+      <c r="A189">
+        <v>2015</v>
+      </c>
+      <c r="B189">
+        <v>0.576181893802856</v>
+      </c>
+      <c r="C189">
+        <v>0.9237840548219957</v>
+      </c>
+      <c r="D189" t="s">
+        <v>20</v>
+      </c>
+      <c r="E189">
+        <v>1365</v>
+      </c>
+      <c r="F189">
+        <v>2501</v>
+      </c>
+      <c r="G189">
+        <v>12190</v>
+      </c>
+    </row>
+    <row r="190" spans="1:7">
+      <c r="A190">
+        <v>2016</v>
+      </c>
+      <c r="B190">
+        <v>0.5699040929352965</v>
+      </c>
+      <c r="C190">
+        <v>0.9315012305168171</v>
+      </c>
+      <c r="D190" t="s">
+        <v>20</v>
+      </c>
+      <c r="E190">
+        <v>1322</v>
+      </c>
+      <c r="F190">
+        <v>2425</v>
+      </c>
+      <c r="G190">
+        <v>12458</v>
+      </c>
+    </row>
+    <row r="191" spans="1:7">
+      <c r="A191">
+        <v>2017</v>
+      </c>
+      <c r="B191">
+        <v>0.3846784104875051</v>
+      </c>
+      <c r="C191">
+        <v>0.9201316423181891</v>
+      </c>
+      <c r="D191" t="s">
+        <v>20</v>
+      </c>
+      <c r="E191">
+        <v>1409</v>
+      </c>
+      <c r="F191">
+        <v>2477</v>
+      </c>
+      <c r="G191">
+        <v>12531</v>
+      </c>
+    </row>
+    <row r="192" spans="1:7">
+      <c r="A192">
+        <v>2018</v>
+      </c>
+      <c r="B192">
+        <v>0.1961405926946933</v>
+      </c>
+      <c r="C192">
+        <v>0.9246668262708483</v>
+      </c>
+      <c r="D192" t="s">
+        <v>20</v>
+      </c>
+      <c r="E192">
+        <v>1506</v>
+      </c>
+      <c r="F192">
+        <v>2421</v>
+      </c>
+      <c r="G192">
+        <v>12502</v>
+      </c>
+    </row>
+    <row r="193" spans="1:7">
+      <c r="A193">
+        <v>2019</v>
+      </c>
+      <c r="B193">
+        <v>0</v>
+      </c>
+      <c r="C193">
+        <v>0.9262517997120461</v>
+      </c>
+      <c r="D193" t="s">
+        <v>20</v>
+      </c>
+      <c r="E193">
+        <v>1344</v>
+      </c>
+      <c r="F193">
+        <v>2357</v>
+      </c>
+      <c r="G193">
+        <v>12593</v>
+      </c>
+    </row>
+    <row r="194" spans="1:7">
+      <c r="A194">
+        <v>2020</v>
+      </c>
+      <c r="B194">
+        <v>0</v>
+      </c>
+      <c r="C194">
+        <v>0.9204319860239816</v>
+      </c>
+      <c r="D194" t="s">
+        <v>20</v>
+      </c>
+      <c r="E194">
+        <v>1360</v>
+      </c>
+      <c r="F194">
+        <v>1453</v>
+      </c>
+      <c r="G194">
+        <v>11684</v>
+      </c>
+    </row>
+    <row r="195" spans="1:7">
+      <c r="A195">
+        <v>2021</v>
+      </c>
+      <c r="B195">
+        <v>0</v>
+      </c>
+      <c r="C195">
+        <v>0.9818555289284492</v>
+      </c>
+      <c r="D195" t="s">
+        <v>20</v>
+      </c>
+      <c r="E195">
+        <v>1402</v>
+      </c>
+      <c r="F195">
+        <v>2489</v>
+      </c>
+      <c r="G195">
+        <v>12559</v>
+      </c>
+    </row>
+    <row r="196" spans="1:7">
+      <c r="A196">
+        <v>2022</v>
+      </c>
+      <c r="B196">
+        <v>0</v>
+      </c>
+      <c r="C196">
+        <v>0.9355840433155506</v>
+      </c>
+      <c r="D196" t="s">
+        <v>20</v>
+      </c>
+      <c r="E196">
+        <v>1394</v>
+      </c>
+      <c r="F196">
+        <v>2477</v>
+      </c>
+      <c r="G196">
+        <v>12833</v>
+      </c>
+    </row>
+    <row r="197" spans="1:7">
+      <c r="A197">
+        <v>2023</v>
+      </c>
+      <c r="B197">
+        <v>0</v>
+      </c>
+      <c r="C197">
+        <v>0.9411673030468324</v>
+      </c>
+      <c r="D197" t="s">
+        <v>20</v>
+      </c>
+      <c r="E197">
+        <v>1423</v>
+      </c>
+      <c r="F197">
+        <v>2794</v>
+      </c>
+      <c r="G197">
+        <v>13449</v>
+      </c>
+    </row>
+    <row r="198" spans="1:7">
+      <c r="A198">
+        <v>2010</v>
+      </c>
+      <c r="B198">
+        <v>3.41025641025641</v>
+      </c>
+      <c r="D198" t="s">
+        <v>21</v>
+      </c>
+      <c r="E198">
+        <v>18</v>
+      </c>
+      <c r="F198">
+        <v>24</v>
+      </c>
+      <c r="G198">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="199" spans="1:7">
+      <c r="A199">
+        <v>2011</v>
+      </c>
+      <c r="B199">
+        <v>2.808510638297872</v>
+      </c>
+      <c r="C199">
+        <v>1.547945205479452</v>
+      </c>
+      <c r="D199" t="s">
+        <v>21</v>
+      </c>
+      <c r="E199">
+        <v>49</v>
+      </c>
+      <c r="F199">
+        <v>15</v>
+      </c>
+      <c r="G199">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="200" spans="1:7">
+      <c r="A200">
+        <v>2012</v>
+      </c>
+      <c r="B200">
+        <v>3.96875</v>
+      </c>
+      <c r="C200">
+        <v>1.265822784810127</v>
+      </c>
+      <c r="D200" t="s">
+        <v>21</v>
+      </c>
+      <c r="E200">
+        <v>39</v>
+      </c>
+      <c r="F200">
+        <v>8</v>
+      </c>
+      <c r="G200">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="201" spans="1:7">
+      <c r="A201">
+        <v>2013</v>
+      </c>
+      <c r="B201">
+        <v>4.310344827586207</v>
+      </c>
+      <c r="C201">
+        <v>1.507246376811594</v>
+      </c>
+      <c r="D201" t="s">
+        <v>21</v>
+      </c>
+      <c r="E201">
+        <v>53</v>
+      </c>
+      <c r="F201">
+        <v>9</v>
+      </c>
+      <c r="G201">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="202" spans="1:7">
+      <c r="A202">
+        <v>2014</v>
+      </c>
+      <c r="B202">
+        <v>3.361111111111111</v>
+      </c>
+      <c r="C202">
+        <v>1.566666666666667</v>
+      </c>
+      <c r="D202" t="s">
+        <v>21</v>
+      </c>
+      <c r="E202">
+        <v>41</v>
+      </c>
+      <c r="F202">
+        <v>12</v>
+      </c>
+      <c r="G202">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="203" spans="1:7">
+      <c r="A203">
+        <v>2015</v>
+      </c>
+      <c r="B203">
+        <v>2.538461538461538</v>
+      </c>
+      <c r="C203">
+        <v>1.307692307692308</v>
+      </c>
+      <c r="D203" t="s">
+        <v>21</v>
+      </c>
+      <c r="E203">
+        <v>41</v>
+      </c>
+      <c r="F203">
+        <v>15</v>
+      </c>
+      <c r="G203">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="204" spans="1:7">
+      <c r="A204">
+        <v>2016</v>
+      </c>
+      <c r="B204">
+        <v>2.03030303030303</v>
+      </c>
+      <c r="C204">
+        <v>1.254237288135593</v>
+      </c>
+      <c r="D204" t="s">
+        <v>21</v>
+      </c>
+      <c r="E204">
+        <v>41</v>
+      </c>
+      <c r="F204">
+        <v>25</v>
+      </c>
+      <c r="G204">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="205" spans="1:7">
+      <c r="A205">
+        <v>2017</v>
+      </c>
+      <c r="B205">
+        <v>1.4</v>
+      </c>
+      <c r="C205">
+        <v>1.931034482758621</v>
+      </c>
+      <c r="D205" t="s">
+        <v>21</v>
+      </c>
+      <c r="E205">
+        <v>51</v>
+      </c>
+      <c r="F205">
+        <v>26</v>
+      </c>
+      <c r="G205">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="206" spans="1:7">
+      <c r="A206">
+        <v>2018</v>
+      </c>
+      <c r="B206">
+        <v>0.8360655737704918</v>
+      </c>
+      <c r="C206">
+        <v>1.413793103448276</v>
+      </c>
+      <c r="D206" t="s">
+        <v>21</v>
+      </c>
+      <c r="E206">
+        <v>40</v>
+      </c>
+      <c r="F206">
+        <v>19</v>
+      </c>
+      <c r="G206">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="207" spans="1:7">
+      <c r="A207">
+        <v>2019</v>
+      </c>
+      <c r="B207">
+        <v>0</v>
+      </c>
+      <c r="C207">
+        <v>1.107843137254902</v>
+      </c>
+      <c r="D207" t="s">
+        <v>21</v>
+      </c>
+      <c r="E207">
+        <v>36</v>
+      </c>
+      <c r="F207">
+        <v>16</v>
+      </c>
+      <c r="G207">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="208" spans="1:7">
+      <c r="A208">
+        <v>2020</v>
+      </c>
+      <c r="B208">
+        <v>0</v>
+      </c>
+      <c r="C208">
+        <v>1.247311827956989</v>
+      </c>
+      <c r="D208" t="s">
+        <v>21</v>
+      </c>
+      <c r="E208">
+        <v>49</v>
+      </c>
+      <c r="F208">
+        <v>39</v>
+      </c>
+      <c r="G208">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="209" spans="1:7">
+      <c r="A209">
+        <v>2021</v>
+      </c>
+      <c r="B209">
+        <v>0</v>
+      </c>
+      <c r="C209">
+        <v>1.047169811320755</v>
+      </c>
+      <c r="D209" t="s">
+        <v>21</v>
+      </c>
+      <c r="E209">
+        <v>36</v>
+      </c>
+      <c r="F209">
+        <v>36</v>
+      </c>
+      <c r="G209">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="210" spans="1:7">
+      <c r="A210">
+        <v>2022</v>
+      </c>
+      <c r="B210">
+        <v>0</v>
+      </c>
+      <c r="C210">
+        <v>1.234234234234234</v>
+      </c>
+      <c r="D210" t="s">
+        <v>21</v>
+      </c>
+      <c r="E210">
+        <v>47</v>
+      </c>
+      <c r="F210">
+        <v>36</v>
+      </c>
+      <c r="G210">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="211" spans="1:7">
+      <c r="A211">
+        <v>2023</v>
+      </c>
+      <c r="B211">
+        <v>0</v>
+      </c>
+      <c r="C211">
+        <v>1.166666666666667</v>
+      </c>
+      <c r="D211" t="s">
+        <v>21</v>
+      </c>
+      <c r="E211">
+        <v>51</v>
+      </c>
+      <c r="F211">
+        <v>28</v>
+      </c>
+      <c r="G211">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="212" spans="1:7">
+      <c r="A212">
+        <v>2010</v>
+      </c>
+      <c r="B212">
+        <v>6.369230769230769</v>
+      </c>
+      <c r="D212" t="s">
+        <v>22</v>
+      </c>
+      <c r="E212">
+        <v>31</v>
+      </c>
+      <c r="F212">
+        <v>39</v>
+      </c>
+      <c r="G212">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="213" spans="1:7">
+      <c r="A213">
+        <v>2011</v>
+      </c>
+      <c r="B213">
+        <v>3.879310344827586</v>
+      </c>
+      <c r="C213">
+        <v>1.45662100456621</v>
+      </c>
+      <c r="D213" t="s">
+        <v>22</v>
+      </c>
+      <c r="E213">
+        <v>121</v>
+      </c>
+      <c r="F213">
+        <v>26</v>
+      </c>
+      <c r="G213">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="214" spans="1:7">
+      <c r="A214">
+        <v>2012</v>
+      </c>
+      <c r="B214">
+        <v>3.359712230215827</v>
+      </c>
+      <c r="C214">
+        <v>1.348214285714286</v>
+      </c>
+      <c r="D214" t="s">
+        <v>22</v>
+      </c>
+      <c r="E214">
+        <v>124</v>
+      </c>
+      <c r="F214">
+        <v>51</v>
+      </c>
+      <c r="G214">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="215" spans="1:7">
+      <c r="A215">
+        <v>2013</v>
+      </c>
+      <c r="B215">
+        <v>3.106666666666666</v>
+      </c>
+      <c r="C215">
+        <v>1.436681222707423</v>
+      </c>
+      <c r="D215" t="s">
+        <v>22</v>
+      </c>
+      <c r="E215">
+        <v>136</v>
+      </c>
+      <c r="F215">
+        <v>62</v>
+      </c>
+      <c r="G215">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="216" spans="1:7">
+      <c r="A216">
+        <v>2014</v>
+      </c>
+      <c r="B216">
+        <v>3.054421768707483</v>
+      </c>
+      <c r="C216">
+        <v>1.270588235294118</v>
+      </c>
+      <c r="D216" t="s">
+        <v>22</v>
+      </c>
+      <c r="E216">
+        <v>136</v>
+      </c>
+      <c r="F216">
+        <v>37</v>
+      </c>
+      <c r="G216">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="217" spans="1:7">
+      <c r="A217">
+        <v>2015</v>
+      </c>
+      <c r="B217">
+        <v>3.171974522292994</v>
+      </c>
+      <c r="C217">
+        <v>1.422222222222222</v>
+      </c>
+      <c r="D217" t="s">
+        <v>22</v>
+      </c>
+      <c r="E217">
+        <v>123</v>
+      </c>
+      <c r="F217">
+        <v>48</v>
+      </c>
+      <c r="G217">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="218" spans="1:7">
+      <c r="A218">
+        <v>2016</v>
+      </c>
+      <c r="B218">
+        <v>3.242937853107345</v>
+      </c>
+      <c r="C218">
+        <v>1.481632653061224</v>
+      </c>
+      <c r="D218" t="s">
+        <v>22</v>
+      </c>
+      <c r="E218">
+        <v>141</v>
+      </c>
+      <c r="F218">
+        <v>72</v>
+      </c>
+      <c r="G218">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="219" spans="1:7">
+      <c r="A219">
+        <v>2017</v>
+      </c>
+      <c r="B219">
+        <v>1.963636363636364</v>
+      </c>
+      <c r="C219">
+        <v>1.30952380952381</v>
+      </c>
+      <c r="D219" t="s">
+        <v>22</v>
+      </c>
+      <c r="E219">
+        <v>150</v>
+      </c>
+      <c r="F219">
+        <v>57</v>
+      </c>
+      <c r="G219">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="220" spans="1:7">
+      <c r="A220">
+        <v>2018</v>
+      </c>
+      <c r="B220">
+        <v>1</v>
+      </c>
+      <c r="C220">
+        <v>1.397260273972603</v>
+      </c>
+      <c r="D220" t="s">
+        <v>22</v>
+      </c>
+      <c r="E220">
+        <v>159</v>
+      </c>
+      <c r="F220">
+        <v>91</v>
+      </c>
+      <c r="G220">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="221" spans="1:7">
+      <c r="A221">
+        <v>2019</v>
+      </c>
+      <c r="B221">
+        <v>0</v>
+      </c>
+      <c r="C221">
+        <v>1.214705882352941</v>
+      </c>
+      <c r="D221" t="s">
+        <v>22</v>
+      </c>
+      <c r="E221">
+        <v>158</v>
+      </c>
+      <c r="F221">
+        <v>77</v>
+      </c>
+      <c r="G221">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="222" spans="1:7">
+      <c r="A222">
+        <v>2020</v>
+      </c>
+      <c r="B222">
+        <v>0</v>
+      </c>
+      <c r="C222">
+        <v>1.283132530120482</v>
+      </c>
+      <c r="D222" t="s">
+        <v>22</v>
+      </c>
+      <c r="E222">
+        <v>149</v>
+      </c>
+      <c r="F222">
+        <v>104</v>
+      </c>
+      <c r="G222">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="223" spans="1:7">
+      <c r="A223">
+        <v>2021</v>
+      </c>
+      <c r="B223">
+        <v>0</v>
+      </c>
+      <c r="C223">
+        <v>1.249343832020997</v>
+      </c>
+      <c r="D223" t="s">
+        <v>22</v>
+      </c>
+      <c r="E223">
+        <v>142</v>
+      </c>
+      <c r="F223">
+        <v>117</v>
+      </c>
+      <c r="G223">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="224" spans="1:7">
+      <c r="A224">
+        <v>2022</v>
+      </c>
+      <c r="B224">
+        <v>0</v>
+      </c>
+      <c r="C224">
+        <v>1.321507760532151</v>
+      </c>
+      <c r="D224" t="s">
+        <v>22</v>
+      </c>
+      <c r="E224">
+        <v>207</v>
+      </c>
+      <c r="F224">
+        <v>113</v>
+      </c>
+      <c r="G224">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="225" spans="1:7">
+      <c r="A225">
+        <v>2023</v>
+      </c>
+      <c r="B225">
+        <v>0</v>
+      </c>
+      <c r="C225">
+        <v>1.258964143426295</v>
+      </c>
+      <c r="D225" t="s">
+        <v>22</v>
+      </c>
+      <c r="E225">
+        <v>225</v>
+      </c>
+      <c r="F225">
+        <v>100</v>
+      </c>
+      <c r="G225">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="226" spans="1:7">
+      <c r="A226">
+        <v>2010</v>
+      </c>
+      <c r="B226">
+        <v>8.266666666666667</v>
+      </c>
+      <c r="D226" t="s">
+        <v>23</v>
+      </c>
+      <c r="E226">
+        <v>33</v>
+      </c>
+      <c r="F226">
+        <v>14</v>
+      </c>
+      <c r="G226">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="227" spans="1:7">
+      <c r="A227">
+        <v>2011</v>
+      </c>
+      <c r="B227">
+        <v>5.882352941176471</v>
+      </c>
+      <c r="C227">
+        <v>1.57843137254902</v>
+      </c>
+      <c r="D227" t="s">
+        <v>23</v>
+      </c>
+      <c r="E227">
+        <v>77</v>
+      </c>
+      <c r="F227">
+        <v>31</v>
+      </c>
+      <c r="G227">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="228" spans="1:7">
+      <c r="A228">
+        <v>2012</v>
+      </c>
+      <c r="B228">
+        <v>5.043956043956044</v>
+      </c>
+      <c r="C228">
+        <v>1.660869565217391</v>
+      </c>
+      <c r="D228" t="s">
+        <v>23</v>
+      </c>
+      <c r="E228">
+        <v>109</v>
+      </c>
+      <c r="F228">
+        <v>23</v>
+      </c>
+      <c r="G228">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="229" spans="1:7">
+      <c r="A229">
+        <v>2013</v>
+      </c>
+      <c r="B229">
+        <v>4.669902912621359</v>
+      </c>
+      <c r="C229">
+        <v>1.790476190476191</v>
+      </c>
+      <c r="D229" t="s">
+        <v>23</v>
+      </c>
+      <c r="E229">
+        <v>97</v>
+      </c>
+      <c r="F229">
+        <v>37</v>
+      </c>
+      <c r="G229">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="230" spans="1:7">
+      <c r="A230">
+        <v>2014</v>
+      </c>
+      <c r="B230">
+        <v>4.556521739130435</v>
+      </c>
+      <c r="C230">
+        <v>1.75</v>
+      </c>
+      <c r="D230" t="s">
+        <v>23</v>
+      </c>
+      <c r="E230">
+        <v>109</v>
+      </c>
+      <c r="F230">
+        <v>43</v>
+      </c>
+      <c r="G230">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="231" spans="1:7">
+      <c r="A231">
+        <v>2015</v>
+      </c>
+      <c r="B231">
+        <v>4.568</v>
+      </c>
+      <c r="C231">
+        <v>1.582278481012658</v>
+      </c>
+      <c r="D231" t="s">
+        <v>23</v>
+      </c>
+      <c r="E231">
+        <v>122</v>
+      </c>
+      <c r="F231">
+        <v>35</v>
+      </c>
+      <c r="G231">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="232" spans="1:7">
+      <c r="A232">
+        <v>2016</v>
+      </c>
+      <c r="B232">
+        <v>4.263513513513513</v>
+      </c>
+      <c r="C232">
+        <v>1.638036809815951</v>
+      </c>
+      <c r="D232" t="s">
+        <v>23</v>
+      </c>
+      <c r="E232">
+        <v>115</v>
+      </c>
+      <c r="F232">
+        <v>47</v>
+      </c>
+      <c r="G232">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="233" spans="1:7">
+      <c r="A233">
+        <v>2017</v>
+      </c>
+      <c r="B233">
+        <v>2.446927374301676</v>
+      </c>
+      <c r="C233">
+        <v>1.457286432160804</v>
+      </c>
+      <c r="D233" t="s">
+        <v>23</v>
+      </c>
+      <c r="E233">
+        <v>135</v>
+      </c>
+      <c r="F233">
+        <v>66</v>
+      </c>
+      <c r="G233">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="234" spans="1:7">
+      <c r="A234">
+        <v>2018</v>
+      </c>
+      <c r="B234">
+        <v>1.079601990049751</v>
+      </c>
+      <c r="C234">
+        <v>1.515837104072398</v>
+      </c>
+      <c r="D234" t="s">
+        <v>23</v>
+      </c>
+      <c r="E234">
+        <v>150</v>
+      </c>
+      <c r="F234">
+        <v>66</v>
+      </c>
+      <c r="G234">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="235" spans="1:7">
+      <c r="A235">
+        <v>2019</v>
+      </c>
+      <c r="B235">
+        <v>0</v>
+      </c>
+      <c r="C235">
+        <v>1.50996015936255</v>
+      </c>
+      <c r="D235" t="s">
+        <v>23</v>
+      </c>
+      <c r="E235">
+        <v>174</v>
+      </c>
+      <c r="F235">
+        <v>69</v>
+      </c>
+      <c r="G235">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="236" spans="1:7">
+      <c r="A236">
+        <v>2020</v>
+      </c>
+      <c r="B236">
+        <v>0</v>
+      </c>
+      <c r="C236">
+        <v>1.354014598540146</v>
+      </c>
+      <c r="D236" t="s">
+        <v>23</v>
+      </c>
+      <c r="E236">
+        <v>157</v>
+      </c>
+      <c r="F236">
+        <v>106</v>
+      </c>
+      <c r="G236">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="237" spans="1:7">
+      <c r="A237">
+        <v>2021</v>
+      </c>
+      <c r="B237">
+        <v>0</v>
+      </c>
+      <c r="C237">
+        <v>1.49375</v>
+      </c>
+      <c r="D237" t="s">
+        <v>23</v>
+      </c>
+      <c r="E237">
+        <v>193</v>
+      </c>
+      <c r="F237">
+        <v>153</v>
+      </c>
+      <c r="G237">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="238" spans="1:7">
+      <c r="A238">
+        <v>2022</v>
+      </c>
+      <c r="B238">
+        <v>0</v>
+      </c>
+      <c r="C238">
+        <v>1.248858447488584</v>
+      </c>
+      <c r="D238" t="s">
+        <v>23</v>
+      </c>
+      <c r="E238">
+        <v>221</v>
+      </c>
+      <c r="F238">
+        <v>91</v>
+      </c>
+      <c r="G238">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="239" spans="1:7">
+      <c r="A239">
+        <v>2023</v>
+      </c>
+      <c r="B239">
+        <v>0</v>
+      </c>
+      <c r="C239">
+        <v>1.290167865707434</v>
+      </c>
+      <c r="D239" t="s">
+        <v>23</v>
+      </c>
+      <c r="E239">
         <v>217</v>
       </c>
-      <c r="F183">
+      <c r="F239">
         <v>111</v>
       </c>
-      <c r="G183">
+      <c r="G239">
         <v>432</v>
       </c>
     </row>

</xml_diff>